<commit_message>
docs(excel): pridané sheets Audity + Daily_audit + Roadmap (v3)
- Audity: 18 audit scriptov s ownerom, frekvenciou, notif chain
- Daily_audit: čo cron sleduje + thresholds + email subjects
- Roadmap: 50 open ticktov (P0-P3) s farebným kódovaním

Excel teraz má 9 sheets, kompletný obraz korporátu.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/vianema-engineering-org.xlsx
+++ b/vianema-engineering-org.xlsx
@@ -12,7 +12,10 @@
     <sheet name="Oddelenia" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Moduly" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Eskalacia" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Denny_rezim" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Audity" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Daily_audit" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Roadmap" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Denny_rezim" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -3790,6 +3793,1345 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:F21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="4" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="38" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>18 audit scriptov — kontrolný systém</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Audit script</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Pre koho</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Frekvencia</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Spúšťa</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Pri fail → notifikácia</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="32" customHeight="1">
+      <c r="A4" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" s="12" t="inlineStr">
+        <is>
+          <t>audit-security.sh</t>
+        </is>
+      </c>
+      <c r="C4" s="12" t="inlineStr">
+        <is>
+          <t>E004 Lukáš (Security Tech Lead)</t>
+        </is>
+      </c>
+      <c r="D4" s="12" t="inlineStr">
+        <is>
+          <t>Pri PR; daily o 02:00</t>
+        </is>
+      </c>
+      <c r="E4" s="12" t="inlineStr">
+        <is>
+          <t>Auto cez audit-all.sh</t>
+        </is>
+      </c>
+      <c r="F4" s="12" t="inlineStr">
+        <is>
+          <t>🚨 Lukáš + Adam + Aleš</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="32" customHeight="1">
+      <c r="A5" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" s="12" t="inlineStr">
+        <is>
+          <t>audit-monitor.sh</t>
+        </is>
+      </c>
+      <c r="C5" s="12" t="inlineStr">
+        <is>
+          <t>E005 Martin (Monitor Tech Lead)</t>
+        </is>
+      </c>
+      <c r="D5" s="12" t="inlineStr">
+        <is>
+          <t>Pri PR; daily o 02:00</t>
+        </is>
+      </c>
+      <c r="E5" s="12" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="F5" s="12" t="inlineStr">
+        <is>
+          <t>🚨 Martin + Patrik</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="32" customHeight="1">
+      <c r="A6" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="B6" s="12" t="inlineStr">
+        <is>
+          <t>audit-klienti.sh</t>
+        </is>
+      </c>
+      <c r="C6" s="12" t="inlineStr">
+        <is>
+          <t>E006 Petra (Klienti Tech Lead)</t>
+        </is>
+      </c>
+      <c r="D6" s="12" t="inlineStr">
+        <is>
+          <t>Pri PR; daily o 02:00</t>
+        </is>
+      </c>
+      <c r="E6" s="12" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="F6" s="12" t="inlineStr">
+        <is>
+          <t>🚨 Petra</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="32" customHeight="1">
+      <c r="A7" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="B7" s="12" t="inlineStr">
+        <is>
+          <t>audit-nehnutelnosti.sh</t>
+        </is>
+      </c>
+      <c r="C7" s="12" t="inlineStr">
+        <is>
+          <t>E007 Andrej (Nehnuteľnosti TL)</t>
+        </is>
+      </c>
+      <c r="D7" s="12" t="inlineStr">
+        <is>
+          <t>Pri PR; daily</t>
+        </is>
+      </c>
+      <c r="E7" s="12" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="F7" s="12" t="inlineStr">
+        <is>
+          <t>🚨 Andrej</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="32" customHeight="1">
+      <c r="A8" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="B8" s="12" t="inlineStr">
+        <is>
+          <t>audit-naberaky.sh</t>
+        </is>
+      </c>
+      <c r="C8" s="12" t="inlineStr">
+        <is>
+          <t>E008 Lenka (Náberáky TL)</t>
+        </is>
+      </c>
+      <c r="D8" s="12" t="inlineStr">
+        <is>
+          <t>Pri PR; daily</t>
+        </is>
+      </c>
+      <c r="E8" s="12" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="F8" s="12" t="inlineStr">
+        <is>
+          <t>🚨 Lenka + Katarína (compliance)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="32" customHeight="1">
+      <c r="A9" s="12" t="n">
+        <v>6</v>
+      </c>
+      <c r="B9" s="12" t="inlineStr">
+        <is>
+          <t>audit-obhliadky.sh</t>
+        </is>
+      </c>
+      <c r="C9" s="12" t="inlineStr">
+        <is>
+          <t>E009 Jozef (Obhliadky TL)</t>
+        </is>
+      </c>
+      <c r="D9" s="12" t="inlineStr">
+        <is>
+          <t>Pri PR; daily</t>
+        </is>
+      </c>
+      <c r="E9" s="12" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="F9" s="12" t="inlineStr">
+        <is>
+          <t>🚨 Jozef</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="32" customHeight="1">
+      <c r="A10" s="12" t="n">
+        <v>7</v>
+      </c>
+      <c r="B10" s="12" t="inlineStr">
+        <is>
+          <t>audit-financie.sh</t>
+        </is>
+      </c>
+      <c r="C10" s="12" t="inlineStr">
+        <is>
+          <t>E010 Mária (Financie TL)</t>
+        </is>
+      </c>
+      <c r="D10" s="12" t="inlineStr">
+        <is>
+          <t>Pri PR; daily</t>
+        </is>
+      </c>
+      <c r="E10" s="12" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="F10" s="12" t="inlineStr">
+        <is>
+          <t>🚨 Mária + Katarína</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="32" customHeight="1">
+      <c r="A11" s="12" t="n">
+        <v>8</v>
+      </c>
+      <c r="B11" s="12" t="inlineStr">
+        <is>
+          <t>audit-google.sh</t>
+        </is>
+      </c>
+      <c r="C11" s="12" t="inlineStr">
+        <is>
+          <t>E011 Roman (Google TL)</t>
+        </is>
+      </c>
+      <c r="D11" s="12" t="inlineStr">
+        <is>
+          <t>Pri PR; daily</t>
+        </is>
+      </c>
+      <c r="E11" s="12" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="F11" s="12" t="inlineStr">
+        <is>
+          <t>🚨 Roman</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="32" customHeight="1">
+      <c r="A12" s="12" t="n">
+        <v>9</v>
+      </c>
+      <c r="B12" s="12" t="inlineStr">
+        <is>
+          <t>audit-ai.sh</t>
+        </is>
+      </c>
+      <c r="C12" s="12" t="inlineStr">
+        <is>
+          <t>E012 Eva (AI TL)</t>
+        </is>
+      </c>
+      <c r="D12" s="12" t="inlineStr">
+        <is>
+          <t>Pri PR; daily</t>
+        </is>
+      </c>
+      <c r="E12" s="12" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="F12" s="12" t="inlineStr">
+        <is>
+          <t>🚨 Eva + Veronika</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="32" customHeight="1">
+      <c r="A13" s="12" t="n">
+        <v>10</v>
+      </c>
+      <c r="B13" s="12" t="inlineStr">
+        <is>
+          <t>audit-operativa.sh</t>
+        </is>
+      </c>
+      <c r="C13" s="12" t="inlineStr">
+        <is>
+          <t>E013 Patrik (Operativa TL)</t>
+        </is>
+      </c>
+      <c r="D13" s="12" t="inlineStr">
+        <is>
+          <t>Pri PR; daily</t>
+        </is>
+      </c>
+      <c r="E13" s="12" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="F13" s="12" t="inlineStr">
+        <is>
+          <t>🚨 Patrik + Michal (SRE)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="32" customHeight="1">
+      <c r="A14" s="12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B14" s="12" t="inlineStr">
+        <is>
+          <t>audit-tests.sh</t>
+        </is>
+      </c>
+      <c r="C14" s="12" t="inlineStr">
+        <is>
+          <t>E014 Daniela (QA)</t>
+        </is>
+      </c>
+      <c r="D14" s="12" t="inlineStr">
+        <is>
+          <t>Pri každom PR (gate)</t>
+        </is>
+      </c>
+      <c r="E14" s="12" t="inlineStr">
+        <is>
+          <t>GitHub Actions</t>
+        </is>
+      </c>
+      <c r="F14" s="12" t="inlineStr">
+        <is>
+          <t>🚨 Daniela + Tech Lead modulu</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="32" customHeight="1">
+      <c r="A15" s="12" t="n">
+        <v>12</v>
+      </c>
+      <c r="B15" s="12" t="inlineStr">
+        <is>
+          <t>audit-perf.sh</t>
+        </is>
+      </c>
+      <c r="C15" s="12" t="inlineStr">
+        <is>
+          <t>E015 Michal (SRE)</t>
+        </is>
+      </c>
+      <c r="D15" s="12" t="inlineStr">
+        <is>
+          <t>Daily + pri PR s perf risk</t>
+        </is>
+      </c>
+      <c r="E15" s="12" t="inlineStr">
+        <is>
+          <t>GitHub Actions + manual</t>
+        </is>
+      </c>
+      <c r="F15" s="12" t="inlineStr">
+        <is>
+          <t>🚨 Michal + Tomáš (CTO)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="32" customHeight="1">
+      <c r="A16" s="12" t="n">
+        <v>13</v>
+      </c>
+      <c r="B16" s="12" t="inlineStr">
+        <is>
+          <t>audit-security-deep.sh</t>
+        </is>
+      </c>
+      <c r="C16" s="12" t="inlineStr">
+        <is>
+          <t>E016 Adam (Sec Auditor)</t>
+        </is>
+      </c>
+      <c r="D16" s="12" t="inlineStr">
+        <is>
+          <t>Týždenne pondelok 04:00</t>
+        </is>
+      </c>
+      <c r="E16" s="12" t="inlineStr">
+        <is>
+          <t>Auto cez audit-all</t>
+        </is>
+      </c>
+      <c r="F16" s="12" t="inlineStr">
+        <is>
+          <t>🚨 Adam + Aleš (priamo CEO)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="32" customHeight="1">
+      <c r="A17" s="12" t="n">
+        <v>14</v>
+      </c>
+      <c r="B17" s="12" t="inlineStr">
+        <is>
+          <t>audit-deploy.sh</t>
+        </is>
+      </c>
+      <c r="C17" s="12" t="inlineStr">
+        <is>
+          <t>E017 Jaroslav (DevOps)</t>
+        </is>
+      </c>
+      <c r="D17" s="12" t="inlineStr">
+        <is>
+          <t>Pri každom deploy</t>
+        </is>
+      </c>
+      <c r="E17" s="12" t="inlineStr">
+        <is>
+          <t>GitHub Actions + manual</t>
+        </is>
+      </c>
+      <c r="F17" s="12" t="inlineStr">
+        <is>
+          <t>🚨 Jaroslav + Tomáš</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="32" customHeight="1">
+      <c r="A18" s="12" t="n">
+        <v>15</v>
+      </c>
+      <c r="B18" s="12" t="inlineStr">
+        <is>
+          <t>audit-compliance.sh</t>
+        </is>
+      </c>
+      <c r="C18" s="12" t="inlineStr">
+        <is>
+          <t>E018 Katarína (Compliance)</t>
+        </is>
+      </c>
+      <c r="D18" s="12" t="inlineStr">
+        <is>
+          <t>Mesačne + pri zmenách PII flow</t>
+        </is>
+      </c>
+      <c r="E18" s="12" t="inlineStr">
+        <is>
+          <t>Manual + audit-all</t>
+        </is>
+      </c>
+      <c r="F18" s="12" t="inlineStr">
+        <is>
+          <t>🚨 Katarína + Aleš (priamo CEO)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="32" customHeight="1">
+      <c r="A19" s="12" t="n">
+        <v>16</v>
+      </c>
+      <c r="B19" s="12" t="inlineStr">
+        <is>
+          <t>audit-content.sh</t>
+        </is>
+      </c>
+      <c r="C19" s="12" t="inlineStr">
+        <is>
+          <t>E019 Veronika (Brand)</t>
+        </is>
+      </c>
+      <c r="D19" s="12" t="inlineStr">
+        <is>
+          <t>Pri každom UI copy zmene</t>
+        </is>
+      </c>
+      <c r="E19" s="12" t="inlineStr">
+        <is>
+          <t>Manual + audit-all</t>
+        </is>
+      </c>
+      <c r="F19" s="12" t="inlineStr">
+        <is>
+          <t>⚠ Veronika</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="32" customHeight="1">
+      <c r="A20" s="12" t="n">
+        <v>17</v>
+      </c>
+      <c r="B20" s="12" t="inlineStr">
+        <is>
+          <t>audit-ui.sh</t>
+        </is>
+      </c>
+      <c r="C20" s="12" t="inlineStr">
+        <is>
+          <t>E020 Šimon (UX)</t>
+        </is>
+      </c>
+      <c r="D20" s="12" t="inlineStr">
+        <is>
+          <t>Pri každom novom komponente</t>
+        </is>
+      </c>
+      <c r="E20" s="12" t="inlineStr">
+        <is>
+          <t>Manual + audit-all</t>
+        </is>
+      </c>
+      <c r="F20" s="12" t="inlineStr">
+        <is>
+          <t>⚠ Šimon</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="32" customHeight="1">
+      <c r="A21" s="12" t="n">
+        <v>18</v>
+      </c>
+      <c r="B21" s="12" t="inlineStr">
+        <is>
+          <t>audit-meta.sh</t>
+        </is>
+      </c>
+      <c r="C21" s="12" t="inlineStr">
+        <is>
+          <t>E023 Mária Hlavatá (IG)</t>
+        </is>
+      </c>
+      <c r="D21" s="12" t="inlineStr">
+        <is>
+          <t>Týždenne piatok 17:00</t>
+        </is>
+      </c>
+      <c r="E21" s="12" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="F21" s="12" t="inlineStr">
+        <is>
+          <t>🚨 Mária H. → CEO</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:F1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="32" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Daily audit cron — čo monitorujeme + komu posiela</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Check</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Kontroluje</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Owner (subagent)</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Threshold pre FAIL</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Email subject prefix</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="40" customHeight="1">
+      <c r="A4" s="12" t="inlineStr">
+        <is>
+          <t>Monitor scrape</t>
+        </is>
+      </c>
+      <c r="B4" s="12" t="inlineStr">
+        <is>
+          <t>Posledný scrape v monitor_inzeraty tabuľke</t>
+        </is>
+      </c>
+      <c r="C4" s="12" t="inlineStr">
+        <is>
+          <t>monitor-owner (Martin + Patrik)</t>
+        </is>
+      </c>
+      <c r="D4" s="12" t="inlineStr">
+        <is>
+          <t>&gt; 36 hodín = FAIL</t>
+        </is>
+      </c>
+      <c r="E4" s="12" t="inlineStr">
+        <is>
+          <t>🚨 Monitor scrape mŕtve</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="40" customHeight="1">
+      <c r="A5" s="12" t="inlineStr">
+        <is>
+          <t>Anon RLS leak</t>
+        </is>
+      </c>
+      <c r="B5" s="12" t="inlineStr">
+        <is>
+          <t>6 privátnych tabuliek: anon dostane data?</t>
+        </is>
+      </c>
+      <c r="C5" s="12" t="inlineStr">
+        <is>
+          <t>security-auditor (Adam + Lukáš)</t>
+        </is>
+      </c>
+      <c r="D5" s="12" t="inlineStr">
+        <is>
+          <t>Anon vidí KTORÚKOĽVEK tabuľku = FAIL</t>
+        </is>
+      </c>
+      <c r="E5" s="12" t="inlineStr">
+        <is>
+          <t>🚨 Anon RLS LEAK</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="40" customHeight="1">
+      <c r="A6" s="12" t="inlineStr">
+        <is>
+          <t>Cron health tracking</t>
+        </is>
+      </c>
+      <c r="B6" s="12" t="inlineStr">
+        <is>
+          <t>Existencia cron_runs tabuľky</t>
+        </is>
+      </c>
+      <c r="C6" s="12" t="inlineStr">
+        <is>
+          <t>operativa-owner (Patrik)</t>
+        </is>
+      </c>
+      <c r="D6" s="12" t="inlineStr">
+        <is>
+          <t>Tabuľka neexistuje = WARN</t>
+        </is>
+      </c>
+      <c r="E6" s="12" t="inlineStr">
+        <is>
+          <t>⚠ Cron health gap</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="40" customHeight="1">
+      <c r="A7" s="12" t="inlineStr">
+        <is>
+          <t>Klient creation activity</t>
+        </is>
+      </c>
+      <c r="B7" s="12" t="inlineStr">
+        <is>
+          <t>Posledný klient_create event</t>
+        </is>
+      </c>
+      <c r="C7" s="12" t="inlineStr">
+        <is>
+          <t>customer-success (Zuzana)</t>
+        </is>
+      </c>
+      <c r="D7" s="12" t="inlineStr">
+        <is>
+          <t>&gt; 14 dní bez nového = WARN</t>
+        </is>
+      </c>
+      <c r="E7" s="12" t="inlineStr">
+        <is>
+          <t>⚠ User activity drop</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="40" customHeight="1">
+      <c r="A8" s="12" t="inlineStr">
+        <is>
+          <t>Google integration</t>
+        </is>
+      </c>
+      <c r="B8" s="12" t="inlineStr">
+        <is>
+          <t>Počet expired Google tokenov</t>
+        </is>
+      </c>
+      <c r="C8" s="12" t="inlineStr">
+        <is>
+          <t>google-owner (Roman)</t>
+        </is>
+      </c>
+      <c r="D8" s="12" t="inlineStr">
+        <is>
+          <t>Akýkoľvek expired = WARN</t>
+        </is>
+      </c>
+      <c r="E8" s="12" t="inlineStr">
+        <is>
+          <t>⚠ Google tokens expire</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>Email logika:</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>• Sektioned: ✓ RESOLVED / 🚨 NEW / ⚠ PERSISTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>• Pošle sa LEN ak diff ≠ unchanged (žiadny spam pri stabilnom stave)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>• Per finding: owner kontakt + subagent ID na aktiváciu v Claude Code</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>• Adresát: ales.machovic@gmail.com (MANAGER_EMAIL)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>• From: noreply@vianema.eu (verified Resend domain)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:E1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D30"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="6" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
+    <col width="35" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Master Roadmap — 50 open ticktov per priorita</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Priorita</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Issue</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="32" customHeight="1">
+      <c r="A4" s="13" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="B4" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="C4" s="13" t="inlineStr">
+        <is>
+          <t>Monitor scrape cron mŕtve 8 dní na vianeme</t>
+        </is>
+      </c>
+      <c r="D4" s="13" t="inlineStr">
+        <is>
+          <t>Martin + Patrik</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="32" customHeight="1">
+      <c r="A5" s="13" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="B5" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="C5" s="13" t="inlineStr">
+        <is>
+          <t>Audit log iba 6% coverage (5/84 routes)</t>
+        </is>
+      </c>
+      <c r="D5" s="13" t="inlineStr">
+        <is>
+          <t>Katarína</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="32" customHeight="1">
+      <c r="A6" s="13" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="B6" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="C6" s="13" t="inlineStr">
+        <is>
+          <t>11 anon RLS USING(true) policies</t>
+        </is>
+      </c>
+      <c r="D6" s="13" t="inlineStr">
+        <is>
+          <t>Adam</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="32" customHeight="1">
+      <c r="A7" s="13" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="B7" s="13" t="n">
+        <v>4</v>
+      </c>
+      <c r="C7" s="13" t="inlineStr">
+        <is>
+          <t>ESLint v9 config rozbitý</t>
+        </is>
+      </c>
+      <c r="D7" s="13" t="inlineStr">
+        <is>
+          <t>Daniela</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="32" customHeight="1">
+      <c r="A8" s="13" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="B8" s="13" t="n">
+        <v>5</v>
+      </c>
+      <c r="C8" s="13" t="inlineStr">
+        <is>
+          <t>ai_usage_log tabuľka chýba</t>
+        </is>
+      </c>
+      <c r="D8" s="13" t="inlineStr">
+        <is>
+          <t>Eva + Mária</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="32" customHeight="1">
+      <c r="A9" s="10" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="B9" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="C9" s="10" t="inlineStr">
+        <is>
+          <t>Pagination na list endpointoch (scale 100 maklerov)</t>
+        </is>
+      </c>
+      <c r="D9" s="10" t="inlineStr">
+        <is>
+          <t>Michal koord</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="32" customHeight="1">
+      <c r="A10" s="10" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="B10" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="C10" s="10" t="inlineStr">
+        <is>
+          <t>Materialized views pre /manazer dashboard</t>
+        </is>
+      </c>
+      <c r="D10" s="10" t="inlineStr">
+        <is>
+          <t>Patrik + Michal</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="32" customHeight="1">
+      <c r="A11" s="10" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="B11" s="10" t="n">
+        <v>8</v>
+      </c>
+      <c r="C11" s="10" t="inlineStr">
+        <is>
+          <t>AML hard blocker pred KZ podpis</t>
+        </is>
+      </c>
+      <c r="D11" s="10" t="inlineStr">
+        <is>
+          <t>Lenka + Katarína</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="32" customHeight="1">
+      <c r="A12" s="10" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="B12" s="10" t="n">
+        <v>9</v>
+      </c>
+      <c r="C12" s="10" t="inlineStr">
+        <is>
+          <t>Reconnect Google OAuth UX</t>
+        </is>
+      </c>
+      <c r="D12" s="10" t="inlineStr">
+        <is>
+          <t>Roman</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="32" customHeight="1">
+      <c r="A13" s="10" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="B13" s="10" t="n">
+        <v>10</v>
+      </c>
+      <c r="C13" s="10" t="inlineStr">
+        <is>
+          <t>30-day device verification</t>
+        </is>
+      </c>
+      <c r="D13" s="10" t="inlineStr">
+        <is>
+          <t>Lukáš</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="32" customHeight="1">
+      <c r="A14" s="10" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="B14" s="10" t="n">
+        <v>11</v>
+      </c>
+      <c r="C14" s="10" t="inlineStr">
+        <is>
+          <t>GitHub Actions CI/CD (TS+test+audit gate)</t>
+        </is>
+      </c>
+      <c r="D14" s="10" t="inlineStr">
+        <is>
+          <t>Jaroslav</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="32" customHeight="1">
+      <c r="A15" s="10" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="B15" s="10" t="n">
+        <v>12</v>
+      </c>
+      <c r="C15" s="10" t="inlineStr">
+        <is>
+          <t>Cron health monitoring tabuľka cron_runs</t>
+        </is>
+      </c>
+      <c r="D15" s="10" t="inlineStr">
+        <is>
+          <t>Patrik</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="32" customHeight="1">
+      <c r="A16" s="10" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="B16" s="10" t="n">
+        <v>13</v>
+      </c>
+      <c r="C16" s="10" t="inlineStr">
+        <is>
+          <t>Password validation min 12+complexity register/reset</t>
+        </is>
+      </c>
+      <c r="D16" s="10" t="inlineStr">
+        <is>
+          <t>Lukáš</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="32" customHeight="1">
+      <c r="A17" s="10" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="B17" s="10" t="n">
+        <v>14</v>
+      </c>
+      <c r="C17" s="10" t="inlineStr">
+        <is>
+          <t>Brand voice blacklist v AI Writer pre-display</t>
+        </is>
+      </c>
+      <c r="D17" s="10" t="inlineStr">
+        <is>
+          <t>Eva + Veronika</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="32" customHeight="1">
+      <c r="A18" s="10" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="B18" s="10" t="n">
+        <v>15</v>
+      </c>
+      <c r="C18" s="10" t="inlineStr">
+        <is>
+          <t>Test coverage pre 8 critical flows</t>
+        </is>
+      </c>
+      <c r="D18" s="10" t="inlineStr">
+        <is>
+          <t>Daniela</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="32" customHeight="1">
+      <c r="A19" s="12" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="B19" s="12" t="n">
+        <v>24</v>
+      </c>
+      <c r="C19" s="12" t="inlineStr">
+        <is>
+          <t>2FA / TOTP pre adminov</t>
+        </is>
+      </c>
+      <c r="D19" s="12" t="inlineStr">
+        <is>
+          <t>Lukáš</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="32" customHeight="1">
+      <c r="A20" s="12" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="B20" s="12" t="n">
+        <v>25</v>
+      </c>
+      <c r="C20" s="12" t="inlineStr">
+        <is>
+          <t>SWR/React Query migrácia</t>
+        </is>
+      </c>
+      <c r="D20" s="12" t="inlineStr">
+        <is>
+          <t>Michal + Tech Leads</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="32" customHeight="1">
+      <c r="A21" s="12" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="B21" s="12" t="n">
+        <v>26</v>
+      </c>
+      <c r="C21" s="12" t="inlineStr">
+        <is>
+          <t>Sec Audit: anon RLS deep scan automated</t>
+        </is>
+      </c>
+      <c r="D21" s="12" t="inlineStr">
+        <is>
+          <t>Adam</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="32" customHeight="1">
+      <c r="A22" s="12" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B22" s="12" t="n">
+        <v>41</v>
+      </c>
+      <c r="C22" s="12" t="inlineStr">
+        <is>
+          <t>RLS sprísnenie z USING(true) na ozajstné policies</t>
+        </is>
+      </c>
+      <c r="D22" s="12" t="inlineStr">
+        <is>
+          <t>Lukáš + Adam</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="32" customHeight="1">
+      <c r="A23" s="12" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B23" s="12" t="n">
+        <v>42</v>
+      </c>
+      <c r="C23" s="12" t="inlineStr">
+        <is>
+          <t>Read replica pre /manazer (Supabase Pro upgrade)</t>
+        </is>
+      </c>
+      <c r="D23" s="12" t="inlineStr">
+        <is>
+          <t>Michal + Jaroslav</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="32" customHeight="1">
+      <c r="A24" s="12" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B24" s="12" t="n">
+        <v>47</v>
+      </c>
+      <c r="C24" s="12" t="inlineStr">
+        <is>
+          <t>Mobile viewport tests v Playwright</t>
+        </is>
+      </c>
+      <c r="D24" s="12" t="inlineStr">
+        <is>
+          <t>Šimon + Daniela</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="6" t="inlineStr">
+        <is>
+          <t>Stav (z memory/roadmap.md):</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>P0 open: 5  |  P1 open: 18  |  P2 open: 17  |  P3 open: 10  |  Total: 50</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Closure rate target: ≥ 50% mesačne (Inspector General tracks)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Sprint review: piatok 16:00 (PM E021 Peter Halás)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:D1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:E24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>

</xml_diff>

<commit_message>
docs(excel): v4 — 3 nové oddelenia (Risk/Data/Vendor) + audit findings sheets
12 sheets celkom:
- Organigram (rozšírený o E024-E026)
- Zamestnanci (26 osôb)
- Oddelenia (14)
- Moduly (10)
- Eskalacia (22 typov)
- Audity (18 scriptov)
- Security_Audit (NEW — 10 findings z pen-test, 5 P0 FIXED)
- Compliance_Gaps (NEW — 12 legal gaps so sankciami)
- Risk_Register (NEW — 20 rizík, top 3 priority, insurance plán)
- Daily_audit
- Roadmap
- Denny_rezim

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/vianema-engineering-org.xlsx
+++ b/vianema-engineering-org.xlsx
@@ -13,9 +13,12 @@
     <sheet name="Moduly" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Eskalacia" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Audity" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Daily_audit" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Roadmap" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Denny_rezim" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Security_Audit" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Compliance_Gaps" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Risk_Register" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Daily_audit" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Roadmap" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Denny_rezim" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -523,7 +526,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D31"/>
+  <dimension ref="A1:D34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1095,9 +1098,1435 @@
         </is>
       </c>
     </row>
+    <row r="32">
+      <c r="A32" s="15" t="inlineStr">
+        <is>
+          <t>L2-IND</t>
+        </is>
+      </c>
+      <c r="B32" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Mgr. Ivana Šebestová</t>
+        </is>
+      </c>
+      <c r="C32" s="15" t="inlineStr">
+        <is>
+          <t>Risk Management (Chief Risk Officer)</t>
+        </is>
+      </c>
+      <c r="D32" s="15" t="inlineStr">
+        <is>
+          <t>Aleš (priamo, nezávislé)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="12" t="inlineStr">
+        <is>
+          <t>L3</t>
+        </is>
+      </c>
+      <c r="B33" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      Ing. Tomáš Klimek</t>
+        </is>
+      </c>
+      <c r="C33" s="12" t="inlineStr">
+        <is>
+          <t>Data Engineering / Analytics</t>
+        </is>
+      </c>
+      <c r="D33" s="12" t="inlineStr">
+        <is>
+          <t>CTO (Tomáš Hrabovský)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="12" t="inlineStr">
+        <is>
+          <t>L3</t>
+        </is>
+      </c>
+      <c r="B34" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      Mgr. Pavol Bardoš</t>
+        </is>
+      </c>
+      <c r="C34" s="12" t="inlineStr">
+        <is>
+          <t>Vendor &amp; Partnership Management</t>
+        </is>
+      </c>
+      <c r="D34" s="12" t="inlineStr">
+        <is>
+          <t>COO (Claude)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:D1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="32" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Daily audit cron — čo monitorujeme + komu posiela</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Check</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Kontroluje</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Owner (subagent)</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Threshold pre FAIL</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Email subject prefix</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="40" customHeight="1">
+      <c r="A4" s="12" t="inlineStr">
+        <is>
+          <t>Monitor scrape</t>
+        </is>
+      </c>
+      <c r="B4" s="12" t="inlineStr">
+        <is>
+          <t>Posledný scrape v monitor_inzeraty tabuľke</t>
+        </is>
+      </c>
+      <c r="C4" s="12" t="inlineStr">
+        <is>
+          <t>monitor-owner (Martin + Patrik)</t>
+        </is>
+      </c>
+      <c r="D4" s="12" t="inlineStr">
+        <is>
+          <t>&gt; 36 hodín = FAIL</t>
+        </is>
+      </c>
+      <c r="E4" s="12" t="inlineStr">
+        <is>
+          <t>🚨 Monitor scrape mŕtve</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="40" customHeight="1">
+      <c r="A5" s="12" t="inlineStr">
+        <is>
+          <t>Anon RLS leak</t>
+        </is>
+      </c>
+      <c r="B5" s="12" t="inlineStr">
+        <is>
+          <t>6 privátnych tabuliek: anon dostane data?</t>
+        </is>
+      </c>
+      <c r="C5" s="12" t="inlineStr">
+        <is>
+          <t>security-auditor (Adam + Lukáš)</t>
+        </is>
+      </c>
+      <c r="D5" s="12" t="inlineStr">
+        <is>
+          <t>Anon vidí KTORÚKOĽVEK tabuľku = FAIL</t>
+        </is>
+      </c>
+      <c r="E5" s="12" t="inlineStr">
+        <is>
+          <t>🚨 Anon RLS LEAK</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="40" customHeight="1">
+      <c r="A6" s="12" t="inlineStr">
+        <is>
+          <t>Cron health tracking</t>
+        </is>
+      </c>
+      <c r="B6" s="12" t="inlineStr">
+        <is>
+          <t>Existencia cron_runs tabuľky</t>
+        </is>
+      </c>
+      <c r="C6" s="12" t="inlineStr">
+        <is>
+          <t>operativa-owner (Patrik)</t>
+        </is>
+      </c>
+      <c r="D6" s="12" t="inlineStr">
+        <is>
+          <t>Tabuľka neexistuje = WARN</t>
+        </is>
+      </c>
+      <c r="E6" s="12" t="inlineStr">
+        <is>
+          <t>⚠ Cron health gap</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="40" customHeight="1">
+      <c r="A7" s="12" t="inlineStr">
+        <is>
+          <t>Klient creation activity</t>
+        </is>
+      </c>
+      <c r="B7" s="12" t="inlineStr">
+        <is>
+          <t>Posledný klient_create event</t>
+        </is>
+      </c>
+      <c r="C7" s="12" t="inlineStr">
+        <is>
+          <t>customer-success (Zuzana)</t>
+        </is>
+      </c>
+      <c r="D7" s="12" t="inlineStr">
+        <is>
+          <t>&gt; 14 dní bez nového = WARN</t>
+        </is>
+      </c>
+      <c r="E7" s="12" t="inlineStr">
+        <is>
+          <t>⚠ User activity drop</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="40" customHeight="1">
+      <c r="A8" s="12" t="inlineStr">
+        <is>
+          <t>Google integration</t>
+        </is>
+      </c>
+      <c r="B8" s="12" t="inlineStr">
+        <is>
+          <t>Počet expired Google tokenov</t>
+        </is>
+      </c>
+      <c r="C8" s="12" t="inlineStr">
+        <is>
+          <t>google-owner (Roman)</t>
+        </is>
+      </c>
+      <c r="D8" s="12" t="inlineStr">
+        <is>
+          <t>Akýkoľvek expired = WARN</t>
+        </is>
+      </c>
+      <c r="E8" s="12" t="inlineStr">
+        <is>
+          <t>⚠ Google tokens expire</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>Email logika:</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>• Sektioned: ✓ RESOLVED / 🚨 NEW / ⚠ PERSISTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>• Pošle sa LEN ak diff ≠ unchanged (žiadny spam pri stabilnom stave)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>• Per finding: owner kontakt + subagent ID na aktiváciu v Claude Code</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>• Adresát: ales.machovic@gmail.com (MANAGER_EMAIL)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>• From: noreply@vianema.eu (verified Resend domain)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:E1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D30"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="6" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
+    <col width="35" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Master Roadmap — 50 open ticktov per priorita</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Priorita</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Issue</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="32" customHeight="1">
+      <c r="A4" s="13" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="B4" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="C4" s="13" t="inlineStr">
+        <is>
+          <t>Monitor scrape cron mŕtve 8 dní na vianeme</t>
+        </is>
+      </c>
+      <c r="D4" s="13" t="inlineStr">
+        <is>
+          <t>Martin + Patrik</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="32" customHeight="1">
+      <c r="A5" s="13" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="B5" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="C5" s="13" t="inlineStr">
+        <is>
+          <t>Audit log iba 6% coverage (5/84 routes)</t>
+        </is>
+      </c>
+      <c r="D5" s="13" t="inlineStr">
+        <is>
+          <t>Katarína</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="32" customHeight="1">
+      <c r="A6" s="13" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="B6" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="C6" s="13" t="inlineStr">
+        <is>
+          <t>11 anon RLS USING(true) policies</t>
+        </is>
+      </c>
+      <c r="D6" s="13" t="inlineStr">
+        <is>
+          <t>Adam</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="32" customHeight="1">
+      <c r="A7" s="13" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="B7" s="13" t="n">
+        <v>4</v>
+      </c>
+      <c r="C7" s="13" t="inlineStr">
+        <is>
+          <t>ESLint v9 config rozbitý</t>
+        </is>
+      </c>
+      <c r="D7" s="13" t="inlineStr">
+        <is>
+          <t>Daniela</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="32" customHeight="1">
+      <c r="A8" s="13" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="B8" s="13" t="n">
+        <v>5</v>
+      </c>
+      <c r="C8" s="13" t="inlineStr">
+        <is>
+          <t>ai_usage_log tabuľka chýba</t>
+        </is>
+      </c>
+      <c r="D8" s="13" t="inlineStr">
+        <is>
+          <t>Eva + Mária</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="32" customHeight="1">
+      <c r="A9" s="10" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="B9" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="C9" s="10" t="inlineStr">
+        <is>
+          <t>Pagination na list endpointoch (scale 100 maklerov)</t>
+        </is>
+      </c>
+      <c r="D9" s="10" t="inlineStr">
+        <is>
+          <t>Michal koord</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="32" customHeight="1">
+      <c r="A10" s="10" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="B10" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="C10" s="10" t="inlineStr">
+        <is>
+          <t>Materialized views pre /manazer dashboard</t>
+        </is>
+      </c>
+      <c r="D10" s="10" t="inlineStr">
+        <is>
+          <t>Patrik + Michal</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="32" customHeight="1">
+      <c r="A11" s="10" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="B11" s="10" t="n">
+        <v>8</v>
+      </c>
+      <c r="C11" s="10" t="inlineStr">
+        <is>
+          <t>AML hard blocker pred KZ podpis</t>
+        </is>
+      </c>
+      <c r="D11" s="10" t="inlineStr">
+        <is>
+          <t>Lenka + Katarína</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="32" customHeight="1">
+      <c r="A12" s="10" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="B12" s="10" t="n">
+        <v>9</v>
+      </c>
+      <c r="C12" s="10" t="inlineStr">
+        <is>
+          <t>Reconnect Google OAuth UX</t>
+        </is>
+      </c>
+      <c r="D12" s="10" t="inlineStr">
+        <is>
+          <t>Roman</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="32" customHeight="1">
+      <c r="A13" s="10" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="B13" s="10" t="n">
+        <v>10</v>
+      </c>
+      <c r="C13" s="10" t="inlineStr">
+        <is>
+          <t>30-day device verification</t>
+        </is>
+      </c>
+      <c r="D13" s="10" t="inlineStr">
+        <is>
+          <t>Lukáš</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="32" customHeight="1">
+      <c r="A14" s="10" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="B14" s="10" t="n">
+        <v>11</v>
+      </c>
+      <c r="C14" s="10" t="inlineStr">
+        <is>
+          <t>GitHub Actions CI/CD (TS+test+audit gate)</t>
+        </is>
+      </c>
+      <c r="D14" s="10" t="inlineStr">
+        <is>
+          <t>Jaroslav</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="32" customHeight="1">
+      <c r="A15" s="10" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="B15" s="10" t="n">
+        <v>12</v>
+      </c>
+      <c r="C15" s="10" t="inlineStr">
+        <is>
+          <t>Cron health monitoring tabuľka cron_runs</t>
+        </is>
+      </c>
+      <c r="D15" s="10" t="inlineStr">
+        <is>
+          <t>Patrik</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="32" customHeight="1">
+      <c r="A16" s="10" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="B16" s="10" t="n">
+        <v>13</v>
+      </c>
+      <c r="C16" s="10" t="inlineStr">
+        <is>
+          <t>Password validation min 12+complexity register/reset</t>
+        </is>
+      </c>
+      <c r="D16" s="10" t="inlineStr">
+        <is>
+          <t>Lukáš</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="32" customHeight="1">
+      <c r="A17" s="10" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="B17" s="10" t="n">
+        <v>14</v>
+      </c>
+      <c r="C17" s="10" t="inlineStr">
+        <is>
+          <t>Brand voice blacklist v AI Writer pre-display</t>
+        </is>
+      </c>
+      <c r="D17" s="10" t="inlineStr">
+        <is>
+          <t>Eva + Veronika</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="32" customHeight="1">
+      <c r="A18" s="10" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="B18" s="10" t="n">
+        <v>15</v>
+      </c>
+      <c r="C18" s="10" t="inlineStr">
+        <is>
+          <t>Test coverage pre 8 critical flows</t>
+        </is>
+      </c>
+      <c r="D18" s="10" t="inlineStr">
+        <is>
+          <t>Daniela</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="32" customHeight="1">
+      <c r="A19" s="12" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="B19" s="12" t="n">
+        <v>24</v>
+      </c>
+      <c r="C19" s="12" t="inlineStr">
+        <is>
+          <t>2FA / TOTP pre adminov</t>
+        </is>
+      </c>
+      <c r="D19" s="12" t="inlineStr">
+        <is>
+          <t>Lukáš</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="32" customHeight="1">
+      <c r="A20" s="12" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="B20" s="12" t="n">
+        <v>25</v>
+      </c>
+      <c r="C20" s="12" t="inlineStr">
+        <is>
+          <t>SWR/React Query migrácia</t>
+        </is>
+      </c>
+      <c r="D20" s="12" t="inlineStr">
+        <is>
+          <t>Michal + Tech Leads</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="32" customHeight="1">
+      <c r="A21" s="12" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="B21" s="12" t="n">
+        <v>26</v>
+      </c>
+      <c r="C21" s="12" t="inlineStr">
+        <is>
+          <t>Sec Audit: anon RLS deep scan automated</t>
+        </is>
+      </c>
+      <c r="D21" s="12" t="inlineStr">
+        <is>
+          <t>Adam</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="32" customHeight="1">
+      <c r="A22" s="12" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B22" s="12" t="n">
+        <v>41</v>
+      </c>
+      <c r="C22" s="12" t="inlineStr">
+        <is>
+          <t>RLS sprísnenie z USING(true) na ozajstné policies</t>
+        </is>
+      </c>
+      <c r="D22" s="12" t="inlineStr">
+        <is>
+          <t>Lukáš + Adam</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="32" customHeight="1">
+      <c r="A23" s="12" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B23" s="12" t="n">
+        <v>42</v>
+      </c>
+      <c r="C23" s="12" t="inlineStr">
+        <is>
+          <t>Read replica pre /manazer (Supabase Pro upgrade)</t>
+        </is>
+      </c>
+      <c r="D23" s="12" t="inlineStr">
+        <is>
+          <t>Michal + Jaroslav</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="32" customHeight="1">
+      <c r="A24" s="12" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B24" s="12" t="n">
+        <v>47</v>
+      </c>
+      <c r="C24" s="12" t="inlineStr">
+        <is>
+          <t>Mobile viewport tests v Playwright</t>
+        </is>
+      </c>
+      <c r="D24" s="12" t="inlineStr">
+        <is>
+          <t>Šimon + Daniela</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="6" t="inlineStr">
+        <is>
+          <t>Stav (z memory/roadmap.md):</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>P0 open: 5  |  P1 open: 18  |  P2 open: 17  |  P3 open: 10  |  Total: 50</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Closure rate target: ≥ 50% mesačne (Inspector General tracks)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Sprint review: piatok 16:00 (PM E021 Peter Halás)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:D1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E24"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
+    <col width="38" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Denný režim — automatizované cron jobs + audit rutiny</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Čas UTC</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Čas SK (UTC+2)</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Akcia</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Kto vykonáva</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Reportuje komu</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="35" customHeight="1">
+      <c r="A4" s="12" t="inlineStr">
+        <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="B4" s="12" t="inlineStr">
+        <is>
+          <t>02:00</t>
+        </is>
+      </c>
+      <c r="C4" s="12" t="inlineStr">
+        <is>
+          <t>Cleanup cron (staré audit záznamy, expired sessions)</t>
+        </is>
+      </c>
+      <c r="D4" s="12" t="inlineStr">
+        <is>
+          <t>Vercel (automatický)</t>
+        </is>
+      </c>
+      <c r="E4" s="12" t="inlineStr">
+        <is>
+          <t>E017 Jaroslav (DevOps)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="35" customHeight="1">
+      <c r="A5" s="12" t="inlineStr">
+        <is>
+          <t>01:00</t>
+        </is>
+      </c>
+      <c r="B5" s="12" t="inlineStr">
+        <is>
+          <t>03:00</t>
+        </is>
+      </c>
+      <c r="C5" s="12" t="inlineStr">
+        <is>
+          <t>Pravidelné náklady — auto-pridanie do prehľadu (0–2 dni pred splatnosťou)</t>
+        </is>
+      </c>
+      <c r="D5" s="12" t="inlineStr">
+        <is>
+          <t>Vercel cron</t>
+        </is>
+      </c>
+      <c r="E5" s="12" t="inlineStr">
+        <is>
+          <t>E010 Mária (Financie)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="35" customHeight="1">
+      <c r="A6" s="12" t="inlineStr">
+        <is>
+          <t>02:00</t>
+        </is>
+      </c>
+      <c r="B6" s="12" t="inlineStr">
+        <is>
+          <t>04:00</t>
+        </is>
+      </c>
+      <c r="C6" s="12" t="inlineStr">
+        <is>
+          <t>Domain audits — všetkých 10 modulov (audit-security.sh, audit-monitor.sh, atď.)</t>
+        </is>
+      </c>
+      <c r="D6" s="12" t="inlineStr">
+        <is>
+          <t>10 Tech Leads (E004-E013)</t>
+        </is>
+      </c>
+      <c r="E6" s="12" t="inlineStr">
+        <is>
+          <t>E003 Tomáš (CTO)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="35" customHeight="1">
+      <c r="A7" s="12" t="inlineStr">
+        <is>
+          <t>03:00</t>
+        </is>
+      </c>
+      <c r="B7" s="12" t="inlineStr">
+        <is>
+          <t>05:00</t>
+        </is>
+      </c>
+      <c r="C7" s="12" t="inlineStr">
+        <is>
+          <t>QA audit — test coverage report, regression status</t>
+        </is>
+      </c>
+      <c r="D7" s="12" t="inlineStr">
+        <is>
+          <t>E014 Daniela</t>
+        </is>
+      </c>
+      <c r="E7" s="12" t="inlineStr">
+        <is>
+          <t>E003 Tomáš (CTO)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="35" customHeight="1">
+      <c r="A8" s="12" t="inlineStr">
+        <is>
+          <t>03:30</t>
+        </is>
+      </c>
+      <c r="B8" s="12" t="inlineStr">
+        <is>
+          <t>05:30</t>
+        </is>
+      </c>
+      <c r="C8" s="12" t="inlineStr">
+        <is>
+          <t>SRE perf benchmark — response time check kritických endpointov</t>
+        </is>
+      </c>
+      <c r="D8" s="12" t="inlineStr">
+        <is>
+          <t>E015 Michal</t>
+        </is>
+      </c>
+      <c r="E8" s="12" t="inlineStr">
+        <is>
+          <t>E003 Tomáš (CTO)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="35" customHeight="1">
+      <c r="A9" s="12" t="inlineStr">
+        <is>
+          <t>04:00</t>
+        </is>
+      </c>
+      <c r="B9" s="12" t="inlineStr">
+        <is>
+          <t>06:00</t>
+        </is>
+      </c>
+      <c r="C9" s="12" t="inlineStr">
+        <is>
+          <t>Security deep scan (PONDELOK týždenne) — anon RLS leak, env audit, pen-test scenáre</t>
+        </is>
+      </c>
+      <c r="D9" s="12" t="inlineStr">
+        <is>
+          <t>E016 Adam (Sec Auditor)</t>
+        </is>
+      </c>
+      <c r="E9" s="12" t="inlineStr">
+        <is>
+          <t>E001 Aleš (CEO)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="35" customHeight="1">
+      <c r="A10" s="12" t="inlineStr">
+        <is>
+          <t>05:00</t>
+        </is>
+      </c>
+      <c r="B10" s="12" t="inlineStr">
+        <is>
+          <t>07:00</t>
+        </is>
+      </c>
+      <c r="C10" s="12" t="inlineStr">
+        <is>
+          <t>Compliance check — GDPR coverage, audit log integrity, faktúra sequence</t>
+        </is>
+      </c>
+      <c r="D10" s="12" t="inlineStr">
+        <is>
+          <t>E018 Katarína</t>
+        </is>
+      </c>
+      <c r="E10" s="12" t="inlineStr">
+        <is>
+          <t>E001 Aleš (CEO)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="35" customHeight="1">
+      <c r="A11" s="12" t="inlineStr">
+        <is>
+          <t>05:00</t>
+        </is>
+      </c>
+      <c r="B11" s="12" t="inlineStr">
+        <is>
+          <t>07:00</t>
+        </is>
+      </c>
+      <c r="C11" s="12" t="inlineStr">
+        <is>
+          <t>Volni klienti cron — 24h dropoff klientov bez aktivity</t>
+        </is>
+      </c>
+      <c r="D11" s="12" t="inlineStr">
+        <is>
+          <t>Vercel cron</t>
+        </is>
+      </c>
+      <c r="E11" s="12" t="inlineStr">
+        <is>
+          <t>E006 Petra (Klienti)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="35" customHeight="1">
+      <c r="A12" s="12" t="inlineStr">
+        <is>
+          <t>06:00</t>
+        </is>
+      </c>
+      <c r="B12" s="12" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="C12" s="12" t="inlineStr">
+        <is>
+          <t>API status cron — healthcheck 3rd party (Anthropic, Gemini, Google, Resend)</t>
+        </is>
+      </c>
+      <c r="D12" s="12" t="inlineStr">
+        <is>
+          <t>Vercel cron</t>
+        </is>
+      </c>
+      <c r="E12" s="12" t="inlineStr">
+        <is>
+          <t>E015 Michal (SRE)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="35" customHeight="1">
+      <c r="A13" s="12" t="inlineStr">
+        <is>
+          <t>06:30</t>
+        </is>
+      </c>
+      <c r="B13" s="12" t="inlineStr">
+        <is>
+          <t>08:30</t>
+        </is>
+      </c>
+      <c r="C13" s="12" t="inlineStr">
+        <is>
+          <t>Daily report email tebe — 'Vianema engineering daily: 8/10 green, 2 warnings'</t>
+        </is>
+      </c>
+      <c r="D13" s="12" t="inlineStr">
+        <is>
+          <t>E002 Claude (orchestrator)</t>
+        </is>
+      </c>
+      <c r="E13" s="12" t="inlineStr">
+        <is>
+          <t>E001 Aleš (CEO)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="35" customHeight="1">
+      <c r="A14" s="12" t="inlineStr">
+        <is>
+          <t>07:00</t>
+        </is>
+      </c>
+      <c r="B14" s="12" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="C14" s="12" t="inlineStr">
+        <is>
+          <t>LV reminder cron — pripomienka pre LV-ká blízko expirácie</t>
+        </is>
+      </c>
+      <c r="D14" s="12" t="inlineStr">
+        <is>
+          <t>Vercel cron</t>
+        </is>
+      </c>
+      <c r="E14" s="12" t="inlineStr">
+        <is>
+          <t>E008 Lenka (Náberáky)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="35" customHeight="1">
+      <c r="A15" s="12" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="B15" s="12" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="C15" s="12" t="inlineStr">
+        <is>
+          <t>Scrape cron (Monitor) — daily fetch z Bazos/Reality/Nehnuteľnosti</t>
+        </is>
+      </c>
+      <c r="D15" s="12" t="inlineStr">
+        <is>
+          <t>Vercel cron</t>
+        </is>
+      </c>
+      <c r="E15" s="12" t="inlineStr">
+        <is>
+          <t>E005 Martin (Monitor)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="35" customHeight="1">
+      <c r="A16" s="12" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="B16" s="12" t="inlineStr">
+        <is>
+          <t>11:00</t>
+        </is>
+      </c>
+      <c r="C16" s="12" t="inlineStr">
+        <is>
+          <t>Monitor-daily — vyhodnocovanie signálov (RELISTED, motivated sellers)</t>
+        </is>
+      </c>
+      <c r="D16" s="12" t="inlineStr">
+        <is>
+          <t>Vercel cron</t>
+        </is>
+      </c>
+      <c r="E16" s="12" t="inlineStr">
+        <is>
+          <t>E005 Martin (Monitor)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="35" customHeight="1">
+      <c r="A17" s="12" t="inlineStr">
+        <is>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="B17" s="12" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="C17" s="12" t="inlineStr">
+        <is>
+          <t>Tím standup (async, zápis v memory/standup.md) — čo robím, čo blokuje</t>
+        </is>
+      </c>
+      <c r="D17" s="12" t="inlineStr">
+        <is>
+          <t>Všetci Tech Leads</t>
+        </is>
+      </c>
+      <c r="E17" s="12" t="inlineStr">
+        <is>
+          <t>E003 Tomáš (CTO)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="35" customHeight="1">
+      <c r="A18" s="12" t="inlineStr">
+        <is>
+          <t>On-demand</t>
+        </is>
+      </c>
+      <c r="B18" s="12" t="inlineStr">
+        <is>
+          <t>On-demand</t>
+        </is>
+      </c>
+      <c r="C18" s="12" t="inlineStr">
+        <is>
+          <t>PR review — pred každým merge</t>
+        </is>
+      </c>
+      <c r="D18" s="12" t="inlineStr">
+        <is>
+          <t>E014 Daniela + Tech Lead + (sec/brand/ux ak relevant)</t>
+        </is>
+      </c>
+      <c r="E18" s="12" t="inlineStr">
+        <is>
+          <t>E002 Claude (COO)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="35" customHeight="1">
+      <c r="A19" s="12" t="inlineStr">
+        <is>
+          <t>Týždenne</t>
+        </is>
+      </c>
+      <c r="B19" s="12" t="inlineStr">
+        <is>
+          <t>PIATOK 16:00</t>
+        </is>
+      </c>
+      <c r="C19" s="12" t="inlineStr">
+        <is>
+          <t>Sprint review + roadmap update — čo sa stalo, čo prichádza</t>
+        </is>
+      </c>
+      <c r="D19" s="12" t="inlineStr">
+        <is>
+          <t>E021 Peter (PM)</t>
+        </is>
+      </c>
+      <c r="E19" s="12" t="inlineStr">
+        <is>
+          <t>E001 Aleš (CEO)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="35" customHeight="1">
+      <c r="A20" s="12" t="inlineStr">
+        <is>
+          <t>Mesačne</t>
+        </is>
+      </c>
+      <c r="B20" s="12" t="inlineStr">
+        <is>
+          <t>1. v mesiaci</t>
+        </is>
+      </c>
+      <c r="C20" s="12" t="inlineStr">
+        <is>
+          <t>Faktúra integrity audit — duplicit, sequence, daň, splatnosť</t>
+        </is>
+      </c>
+      <c r="D20" s="12" t="inlineStr">
+        <is>
+          <t>E010 Mária + E018 Katarína</t>
+        </is>
+      </c>
+      <c r="E20" s="12" t="inlineStr">
+        <is>
+          <t>E001 Aleš (CEO)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="35" customHeight="1">
+      <c r="A21" s="12" t="inlineStr">
+        <is>
+          <t>Kvartálne</t>
+        </is>
+      </c>
+      <c r="B21" s="12" t="inlineStr">
+        <is>
+          <t>1. deň kvartálu</t>
+        </is>
+      </c>
+      <c r="C21" s="12" t="inlineStr">
+        <is>
+          <t>Security health report — známkovanie všetkých 10 domén</t>
+        </is>
+      </c>
+      <c r="D21" s="12" t="inlineStr">
+        <is>
+          <t>E016 Adam (Sec Auditor)</t>
+        </is>
+      </c>
+      <c r="E21" s="12" t="inlineStr">
+        <is>
+          <t>E001 Aleš (CEO)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="35" customHeight="1">
+      <c r="A22" s="15" t="inlineStr">
+        <is>
+          <t>01:30</t>
+        </is>
+      </c>
+      <c r="B22" s="15" t="inlineStr">
+        <is>
+          <t>03:30</t>
+        </is>
+      </c>
+      <c r="C22" s="15" t="inlineStr">
+        <is>
+          <t>Meta audit (memory rot, audit script freshness) — Inspector General</t>
+        </is>
+      </c>
+      <c r="D22" s="15" t="inlineStr">
+        <is>
+          <t>E023 Mária (IG)</t>
+        </is>
+      </c>
+      <c r="E22" s="15" t="inlineStr">
+        <is>
+          <t>E002 Claude (COO)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="35" customHeight="1">
+      <c r="A23" s="15" t="inlineStr">
+        <is>
+          <t>Týždenne</t>
+        </is>
+      </c>
+      <c r="B23" s="15" t="inlineStr">
+        <is>
+          <t>PIATOK 17:00</t>
+        </is>
+      </c>
+      <c r="C23" s="15" t="inlineStr">
+        <is>
+          <t>Internal audit report — kto nerobí svoju prácu, TODO trends, kritické nálezy</t>
+        </is>
+      </c>
+      <c r="D23" s="15" t="inlineStr">
+        <is>
+          <t>E023 Mária (IG)</t>
+        </is>
+      </c>
+      <c r="E23" s="15" t="inlineStr">
+        <is>
+          <t>E001 Aleš (CEO)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="35" customHeight="1">
+      <c r="A24" s="15" t="inlineStr">
+        <is>
+          <t>Mesačne</t>
+        </is>
+      </c>
+      <c r="B24" s="15" t="inlineStr">
+        <is>
+          <t>1. v mesiaci</t>
+        </is>
+      </c>
+      <c r="C24" s="15" t="inlineStr">
+        <is>
+          <t>Aggregate external watch sources reports (čo nové v práve, security, AI atď.)</t>
+        </is>
+      </c>
+      <c r="D24" s="15" t="inlineStr">
+        <is>
+          <t>E023 + Katarína + Adam + ostatní</t>
+        </is>
+      </c>
+      <c r="E24" s="15" t="inlineStr">
+        <is>
+          <t>E001 Aleš (CEO)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:E1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1109,7 +2538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H26"/>
+  <dimension ref="A1:H29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1814,7 +3243,7 @@
       </c>
       <c r="C19" s="12" t="inlineStr">
         <is>
-          <t>Security Auditor (nezávislý)</t>
+          <t>Security Auditor (Pen-tester, ex-bankár OSCP/CEH)</t>
         </is>
       </c>
       <c r="D19" s="12" t="inlineStr">
@@ -1829,7 +3258,7 @@
       </c>
       <c r="F19" s="12" t="inlineStr">
         <is>
-          <t>Cross-cutting — independent security review, pen-test mindset, RLS audit</t>
+          <t>PEN-TESTER mindset: ako najlepší hacker. 10 attack scenárov týždenne (anon RLS, cross-tenant, token forge, SSRF, supply chain). Banková úroveň. 5 threat aktérov (kriminálnik, konkurencia, štát, GDPR aktivist, insider).</t>
         </is>
       </c>
       <c r="G19" s="12" t="inlineStr">
@@ -2134,6 +3563,132 @@
       <c r="H26" s="15" t="inlineStr">
         <is>
           <t>Memory rot, audit script nebehol &gt; 14d, TODO closure rate &lt; 30%, kritický fail nezaadresovaný &gt; 7d</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="70" customHeight="1">
+      <c r="A27" s="15" t="inlineStr">
+        <is>
+          <t>E024</t>
+        </is>
+      </c>
+      <c r="B27" s="15" t="inlineStr">
+        <is>
+          <t>Mgr. Ivana Šebestová</t>
+        </is>
+      </c>
+      <c r="C27" s="15" t="inlineStr">
+        <is>
+          <t>Chief Risk Officer (CRO)</t>
+        </is>
+      </c>
+      <c r="D27" s="15" t="inlineStr">
+        <is>
+          <t>Risk Management</t>
+        </is>
+      </c>
+      <c r="E27" s="15" t="inlineStr">
+        <is>
+          <t>E001 (direct, nezávislé)</t>
+        </is>
+      </c>
+      <c r="F27" s="15" t="inlineStr">
+        <is>
+          <t>Risk register (4 kategórie), FRM metodika, insurance, disaster recovery, RTO/RPO</t>
+        </is>
+      </c>
+      <c r="G27" s="15" t="inlineStr">
+        <is>
+          <t>Týždenne risk register refresh; kvartálne CEO review</t>
+        </is>
+      </c>
+      <c r="H27" s="15" t="inlineStr">
+        <is>
+          <t>Pri novom rizku, vendor outage, regulatory zmene, finančný anomálii — Telegram CEO</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="70" customHeight="1">
+      <c r="A28" s="15" t="inlineStr">
+        <is>
+          <t>E025</t>
+        </is>
+      </c>
+      <c r="B28" s="15" t="inlineStr">
+        <is>
+          <t>Ing. Tomáš Klimek</t>
+        </is>
+      </c>
+      <c r="C28" s="15" t="inlineStr">
+        <is>
+          <t>Lead Data Engineer</t>
+        </is>
+      </c>
+      <c r="D28" s="15" t="inlineStr">
+        <is>
+          <t>Data Engineering</t>
+        </is>
+      </c>
+      <c r="E28" s="15" t="inlineStr">
+        <is>
+          <t>E003 CTO</t>
+        </is>
+      </c>
+      <c r="F28" s="15" t="inlineStr">
+        <is>
+          <t>Materialized views, ETL, BI tools, data quality, /manazer dashboard</t>
+        </is>
+      </c>
+      <c r="G28" s="15" t="inlineStr">
+        <is>
+          <t>Mesačne dashboard refresh, priebežne data quality monitoring</t>
+        </is>
+      </c>
+      <c r="H28" s="15" t="inlineStr">
+        <is>
+          <t>Pri perf probléme na dashboardoch, dáta dropping, anomaly detection</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="70" customHeight="1">
+      <c r="A29" s="15" t="inlineStr">
+        <is>
+          <t>E026</t>
+        </is>
+      </c>
+      <c r="B29" s="15" t="inlineStr">
+        <is>
+          <t>Mgr. Pavol Bardoš</t>
+        </is>
+      </c>
+      <c r="C29" s="15" t="inlineStr">
+        <is>
+          <t>Vendor &amp; Partnership Manager</t>
+        </is>
+      </c>
+      <c r="D29" s="15" t="inlineStr">
+        <is>
+          <t>Vendor Management</t>
+        </is>
+      </c>
+      <c r="E29" s="15" t="inlineStr">
+        <is>
+          <t>E002 COO</t>
+        </is>
+      </c>
+      <c r="F29" s="15" t="inlineStr">
+        <is>
+          <t>10 vendor register, DPA tracking, cost monitoring, SLA breach playbook, contract renewals</t>
+        </is>
+      </c>
+      <c r="G29" s="15" t="inlineStr">
+        <is>
+          <t>Týždenne vendor status check, mesačne cost review</t>
+        </is>
+      </c>
+      <c r="H29" s="15" t="inlineStr">
+        <is>
+          <t>Vendor outage, cost spike, DPA expiry, renewal upcoming</t>
         </is>
       </c>
     </row>
@@ -2151,7 +3706,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G15"/>
+  <dimension ref="A1:G18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -2648,6 +4203,117 @@
       <c r="G15" s="15" t="inlineStr">
         <is>
           <t>.claude/agents/inspector-general.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="55" customHeight="1">
+      <c r="A16" s="15" t="inlineStr">
+        <is>
+          <t>Risk Management</t>
+        </is>
+      </c>
+      <c r="B16" s="15" t="inlineStr">
+        <is>
+          <t>Mgr. Ivana Šebestová (E024)</t>
+        </is>
+      </c>
+      <c r="C16" s="15" t="inlineStr">
+        <is>
+          <t>E024</t>
+        </is>
+      </c>
+      <c r="D16" s="15" t="inlineStr">
+        <is>
+          <t>4 kategórie rizík (operačné, finančné, compliance, reputačné), top 20 risk register, insurance recommendations, disaster recovery plan</t>
+        </is>
+      </c>
+      <c r="E16" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F16" s="15" t="inlineStr">
+        <is>
+          <t>memory/role-risk-management.md</t>
+        </is>
+      </c>
+      <c r="G16" s="15" t="inlineStr">
+        <is>
+          <t>.claude/agents/ (TBD)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="55" customHeight="1">
+      <c r="A17" s="15" t="inlineStr">
+        <is>
+          <t>Data Engineering</t>
+        </is>
+      </c>
+      <c r="B17" s="15" t="inlineStr">
+        <is>
+          <t>Ing. Tomáš Klimek (E025)</t>
+        </is>
+      </c>
+      <c r="C17" s="15" t="inlineStr">
+        <is>
+          <t>E025</t>
+        </is>
+      </c>
+      <c r="D17" s="15" t="inlineStr">
+        <is>
+          <t>Materialized views pre /manazer, ETL pipeline, data quality, BI tool evaluation, anomaly detection</t>
+        </is>
+      </c>
+      <c r="E17" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F17" s="15" t="inlineStr">
+        <is>
+          <t>memory/role-data-engineering.md</t>
+        </is>
+      </c>
+      <c r="G17" s="15" t="inlineStr">
+        <is>
+          <t>.claude/agents/ (TBD)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="55" customHeight="1">
+      <c r="A18" s="15" t="inlineStr">
+        <is>
+          <t>Vendor Management</t>
+        </is>
+      </c>
+      <c r="B18" s="15" t="inlineStr">
+        <is>
+          <t>Mgr. Pavol Bardoš (E026)</t>
+        </is>
+      </c>
+      <c r="C18" s="15" t="inlineStr">
+        <is>
+          <t>E026</t>
+        </is>
+      </c>
+      <c r="D18" s="15" t="inlineStr">
+        <is>
+          <t>10 vendor register, DPA compliance tracking, cost monitoring, SLA breach playbook, renewal management</t>
+        </is>
+      </c>
+      <c r="E18" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F18" s="15" t="inlineStr">
+        <is>
+          <t>memory/role-vendor-management.md</t>
+        </is>
+      </c>
+      <c r="G18" s="15" t="inlineStr">
+        <is>
+          <t>.claude/agents/ (TBD)</t>
         </is>
       </c>
     </row>
@@ -4397,230 +6063,359 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:F13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="42" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
-    <col width="32" customWidth="1" min="5" max="5"/>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="52" customWidth="1" min="3" max="3"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Daily audit cron — čo monitorujeme + komu posiela</t>
+          <t>Security pen-test audit 2026-05-19 — 5 P0 fixes + 5 P1</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Check</t>
+          <t>#</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Kontroluje</t>
+          <t>Severity</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Owner (subagent)</t>
+          <t>Issue</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Threshold pre FAIL</t>
+          <t>Location</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Email subject prefix</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="40" customHeight="1">
-      <c r="A4" s="12" t="inlineStr">
-        <is>
-          <t>Monitor scrape</t>
-        </is>
-      </c>
-      <c r="B4" s="12" t="inlineStr">
-        <is>
-          <t>Posledný scrape v monitor_inzeraty tabuľke</t>
-        </is>
-      </c>
-      <c r="C4" s="12" t="inlineStr">
-        <is>
-          <t>monitor-owner (Martin + Patrik)</t>
-        </is>
-      </c>
-      <c r="D4" s="12" t="inlineStr">
-        <is>
-          <t>&gt; 36 hodín = FAIL</t>
-        </is>
-      </c>
-      <c r="E4" s="12" t="inlineStr">
-        <is>
-          <t>🚨 Monitor scrape mŕtve</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="40" customHeight="1">
-      <c r="A5" s="12" t="inlineStr">
-        <is>
-          <t>Anon RLS leak</t>
-        </is>
-      </c>
-      <c r="B5" s="12" t="inlineStr">
-        <is>
-          <t>6 privátnych tabuliek: anon dostane data?</t>
-        </is>
-      </c>
-      <c r="C5" s="12" t="inlineStr">
-        <is>
-          <t>security-auditor (Adam + Lukáš)</t>
-        </is>
-      </c>
-      <c r="D5" s="12" t="inlineStr">
-        <is>
-          <t>Anon vidí KTORÚKOĽVEK tabuľku = FAIL</t>
-        </is>
-      </c>
-      <c r="E5" s="12" t="inlineStr">
-        <is>
-          <t>🚨 Anon RLS LEAK</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="40" customHeight="1">
-      <c r="A6" s="12" t="inlineStr">
-        <is>
-          <t>Cron health tracking</t>
-        </is>
-      </c>
-      <c r="B6" s="12" t="inlineStr">
-        <is>
-          <t>Existencia cron_runs tabuľky</t>
-        </is>
-      </c>
-      <c r="C6" s="12" t="inlineStr">
-        <is>
-          <t>operativa-owner (Patrik)</t>
-        </is>
-      </c>
-      <c r="D6" s="12" t="inlineStr">
-        <is>
-          <t>Tabuľka neexistuje = WARN</t>
-        </is>
-      </c>
-      <c r="E6" s="12" t="inlineStr">
-        <is>
-          <t>⚠ Cron health gap</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="40" customHeight="1">
-      <c r="A7" s="12" t="inlineStr">
-        <is>
-          <t>Klient creation activity</t>
-        </is>
-      </c>
-      <c r="B7" s="12" t="inlineStr">
-        <is>
-          <t>Posledný klient_create event</t>
-        </is>
-      </c>
-      <c r="C7" s="12" t="inlineStr">
-        <is>
-          <t>customer-success (Zuzana)</t>
-        </is>
-      </c>
-      <c r="D7" s="12" t="inlineStr">
-        <is>
-          <t>&gt; 14 dní bez nového = WARN</t>
-        </is>
-      </c>
-      <c r="E7" s="12" t="inlineStr">
-        <is>
-          <t>⚠ User activity drop</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="40" customHeight="1">
-      <c r="A8" s="12" t="inlineStr">
-        <is>
-          <t>Google integration</t>
-        </is>
-      </c>
-      <c r="B8" s="12" t="inlineStr">
-        <is>
-          <t>Počet expired Google tokenov</t>
-        </is>
-      </c>
-      <c r="C8" s="12" t="inlineStr">
-        <is>
-          <t>google-owner (Roman)</t>
-        </is>
-      </c>
-      <c r="D8" s="12" t="inlineStr">
-        <is>
-          <t>Akýkoľvek expired = WARN</t>
-        </is>
-      </c>
-      <c r="E8" s="12" t="inlineStr">
-        <is>
-          <t>⚠ Google tokens expire</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="6" t="inlineStr">
-        <is>
-          <t>Email logika:</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>• Sektioned: ✓ RESOLVED / 🚨 NEW / ⚠ PERSISTENT</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>• Pošle sa LEN ak diff ≠ unchanged (žiadny spam pri stabilnom stave)</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>• Per finding: owner kontakt + subagent ID na aktiváciu v Claude Code</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>• Adresát: ales.machovic@gmail.com (MANAGER_EMAIL)</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>• From: noreply@vianema.eu (verified Resend domain)</t>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Fix commit</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="38" customHeight="1">
+      <c r="A4" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" s="11" t="inlineStr">
+        <is>
+          <t>P0 CRITICAL</t>
+        </is>
+      </c>
+      <c r="C4" s="11" t="inlineStr">
+        <is>
+          <t>session-bootstrap mintne admin session bez hesla</t>
+        </is>
+      </c>
+      <c r="D4" s="11" t="inlineStr">
+        <is>
+          <t>src/app/api/auth/session-bootstrap/route.ts</t>
+        </is>
+      </c>
+      <c r="E4" s="11" t="inlineStr">
+        <is>
+          <t>✅ FIXED (410 Gone)</t>
+        </is>
+      </c>
+      <c r="F4" s="11" t="inlineStr">
+        <is>
+          <t>a1854d8</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="38" customHeight="1">
+      <c r="A5" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" s="11" t="inlineStr">
+        <is>
+          <t>P0 CRITICAL</t>
+        </is>
+      </c>
+      <c r="C5" s="11" t="inlineStr">
+        <is>
+          <t>Open registration s admin role + cudzia company</t>
+        </is>
+      </c>
+      <c r="D5" s="11" t="inlineStr">
+        <is>
+          <t>src/app/api/auth/register/route.ts</t>
+        </is>
+      </c>
+      <c r="E5" s="11" t="inlineStr">
+        <is>
+          <t>✅ FIXED (SIGNUP_ENABLED flag)</t>
+        </is>
+      </c>
+      <c r="F5" s="11" t="inlineStr">
+        <is>
+          <t>a1854d8</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="38" customHeight="1">
+      <c r="A6" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="B6" s="11" t="inlineStr">
+        <is>
+          <t>P0 CRITICAL</t>
+        </is>
+      </c>
+      <c r="C6" s="11" t="inlineStr">
+        <is>
+          <t>Anyone resetne admin password</t>
+        </is>
+      </c>
+      <c r="D6" s="11" t="inlineStr">
+        <is>
+          <t>src/app/api/users/reset-password/route.ts</t>
+        </is>
+      </c>
+      <c r="E6" s="11" t="inlineStr">
+        <is>
+          <t>✅ FIXED (requireUser + admin)</t>
+        </is>
+      </c>
+      <c r="F6" s="11" t="inlineStr">
+        <is>
+          <t>a1854d8</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="38" customHeight="1">
+      <c r="A7" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="B7" s="11" t="inlineStr">
+        <is>
+          <t>P0 CRITICAL</t>
+        </is>
+      </c>
+      <c r="C7" s="11" t="inlineStr">
+        <is>
+          <t>Anon RLS full CRUD na obchody/obhliadky/klient_udalosti</t>
+        </is>
+      </c>
+      <c r="D7" s="11" t="inlineStr">
+        <is>
+          <t>supabase RLS policies</t>
+        </is>
+      </c>
+      <c r="E7" s="11" t="inlineStr">
+        <is>
+          <t>✅ FIXED (migrácia 072)</t>
+        </is>
+      </c>
+      <c r="F7" s="11" t="inlineStr">
+        <is>
+          <t>a1854d8</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="38" customHeight="1">
+      <c r="A8" s="11" t="n">
+        <v>5</v>
+      </c>
+      <c r="B8" s="11" t="inlineStr">
+        <is>
+          <t>P0 CRITICAL</t>
+        </is>
+      </c>
+      <c r="C8" s="11" t="inlineStr">
+        <is>
+          <t>SSRF cez /api/analyze-url — AWS metadata exploit</t>
+        </is>
+      </c>
+      <c r="D8" s="11" t="inlineStr">
+        <is>
+          <t>src/app/api/analyze-url/route.ts</t>
+        </is>
+      </c>
+      <c r="E8" s="11" t="inlineStr">
+        <is>
+          <t>✅ FIXED (auth + URL allowlist)</t>
+        </is>
+      </c>
+      <c r="F8" s="11" t="inlineStr">
+        <is>
+          <t>06422e5</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="38" customHeight="1">
+      <c r="A9" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="B9" s="10" t="inlineStr">
+        <is>
+          <t>P1 HIGH</t>
+        </is>
+      </c>
+      <c r="C9" s="10" t="inlineStr">
+        <is>
+          <t>Cross-tenant leak /api/users + /api/makleri</t>
+        </is>
+      </c>
+      <c r="D9" s="10" t="inlineStr">
+        <is>
+          <t>src/app/api/users/route.ts:17</t>
+        </is>
+      </c>
+      <c r="E9" s="10" t="inlineStr">
+        <is>
+          <t>🟡 TODO</t>
+        </is>
+      </c>
+      <c r="F9" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="38" customHeight="1">
+      <c r="A10" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="B10" s="10" t="inlineStr">
+        <is>
+          <t>P1 HIGH</t>
+        </is>
+      </c>
+      <c r="C10" s="10" t="inlineStr">
+        <is>
+          <t>File upload DoS — parse-doc bez size limit</t>
+        </is>
+      </c>
+      <c r="D10" s="10" t="inlineStr">
+        <is>
+          <t>src/app/api/parse-doc/route.ts</t>
+        </is>
+      </c>
+      <c r="E10" s="10" t="inlineStr">
+        <is>
+          <t>🟡 TODO</t>
+        </is>
+      </c>
+      <c r="F10" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="38" customHeight="1">
+      <c r="A11" s="12" t="n">
+        <v>8</v>
+      </c>
+      <c r="B11" s="12" t="inlineStr">
+        <is>
+          <t>P2 MEDIUM</t>
+        </is>
+      </c>
+      <c r="C11" s="12" t="inlineStr">
+        <is>
+          <t>Session SESSION_SECRET fallback weak</t>
+        </is>
+      </c>
+      <c r="D11" s="12" t="inlineStr">
+        <is>
+          <t>src/lib/auth/session.ts:32-46</t>
+        </is>
+      </c>
+      <c r="E11" s="12" t="inlineStr">
+        <is>
+          <t>🟡 TODO</t>
+        </is>
+      </c>
+      <c r="F11" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="38" customHeight="1">
+      <c r="A12" s="11" t="n">
+        <v>9</v>
+      </c>
+      <c r="B12" s="11" t="inlineStr">
+        <is>
+          <t>P2 MEDIUM</t>
+        </is>
+      </c>
+      <c r="C12" s="11" t="inlineStr">
+        <is>
+          <t>Password policy 8 chars (invariant: 12+complexity)</t>
+        </is>
+      </c>
+      <c r="D12" s="11" t="inlineStr">
+        <is>
+          <t>src/lib/auth/password.ts:5</t>
+        </is>
+      </c>
+      <c r="E12" s="11" t="inlineStr">
+        <is>
+          <t>✅ FIXED (register fix)</t>
+        </is>
+      </c>
+      <c r="F12" s="11" t="inlineStr">
+        <is>
+          <t>a1854d8</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="38" customHeight="1">
+      <c r="A13" s="12" t="n">
+        <v>10</v>
+      </c>
+      <c r="B13" s="12" t="inlineStr">
+        <is>
+          <t>P2 MEDIUM</t>
+        </is>
+      </c>
+      <c r="C13" s="12" t="inlineStr">
+        <is>
+          <t>XSS risk: 3 súborov dangerouslySetInnerHTML</t>
+        </is>
+      </c>
+      <c r="D13" s="12" t="inlineStr">
+        <is>
+          <t>src/app/layout.tsx + 2 ďalšie</t>
+        </is>
+      </c>
+      <c r="E13" s="12" t="inlineStr">
+        <is>
+          <t>🟡 TODO</t>
+        </is>
+      </c>
+      <c r="F13" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A1:F1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4632,495 +6427,443 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D30"/>
+  <dimension ref="A1:F15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="6" customWidth="1" min="2" max="2"/>
-    <col width="60" customWidth="1" min="3" max="3"/>
-    <col width="35" customWidth="1" min="4" max="4"/>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="50" customWidth="1" min="3" max="3"/>
+    <col width="32" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Master Roadmap — 50 open ticktov per priorita</t>
+          <t>Compliance gaps — SK zákony 2026 + audit</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Priorita</t>
+          <t>#</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>#</t>
+          <t>Zákon / norma</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Issue</t>
+          <t>Gap</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
+          <t>Aktuálna sankcia (EUR)</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
           <t>Owner</t>
         </is>
       </c>
-    </row>
-    <row r="4" ht="32" customHeight="1">
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Deadline</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="40" customHeight="1">
       <c r="A4" s="13" t="inlineStr">
         <is>
-          <t>P0</t>
-        </is>
-      </c>
-      <c r="B4" s="13" t="n">
-        <v>1</v>
+          <t>A1</t>
+        </is>
+      </c>
+      <c r="B4" s="13" t="inlineStr">
+        <is>
+          <t>AML zákon 73/2026 § 50</t>
+        </is>
       </c>
       <c r="C4" s="13" t="inlineStr">
         <is>
-          <t>Monitor scrape cron mŕtve 8 dní na vianeme</t>
+          <t>VIANEMA NEzaregistrovaná ako povinná osoba</t>
         </is>
       </c>
       <c r="D4" s="13" t="inlineStr">
         <is>
-          <t>Martin + Patrik</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="32" customHeight="1">
+          <t>165 000 + zákaz činnosti</t>
+        </is>
+      </c>
+      <c r="E4" s="13" t="inlineStr">
+        <is>
+          <t>Katarína (E018)</t>
+        </is>
+      </c>
+      <c r="F4" s="13" t="inlineStr">
+        <is>
+          <t>**31.8.2026 zákon**</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="40" customHeight="1">
       <c r="A5" s="13" t="inlineStr">
         <is>
-          <t>P0</t>
-        </is>
-      </c>
-      <c r="B5" s="13" t="n">
-        <v>2</v>
+          <t>A2</t>
+        </is>
+      </c>
+      <c r="B5" s="13" t="inlineStr">
+        <is>
+          <t>DPH § 76 + ZoÚ § 35</t>
+        </is>
       </c>
       <c r="C5" s="13" t="inlineStr">
         <is>
-          <t>Audit log iba 6% coverage (5/84 routes)</t>
+          <t>Faktúry sa fyzicky mažú (retention 10y porušená)</t>
         </is>
       </c>
       <c r="D5" s="13" t="inlineStr">
         <is>
-          <t>Katarína</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="32" customHeight="1">
-      <c r="A6" s="13" t="inlineStr">
-        <is>
-          <t>P0</t>
-        </is>
-      </c>
-      <c r="B6" s="13" t="n">
-        <v>3</v>
-      </c>
-      <c r="C6" s="13" t="inlineStr">
-        <is>
-          <t>11 anon RLS USING(true) policies</t>
-        </is>
-      </c>
-      <c r="D6" s="13" t="inlineStr">
-        <is>
-          <t>Adam</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="32" customHeight="1">
-      <c r="A7" s="13" t="inlineStr">
-        <is>
-          <t>P0</t>
-        </is>
-      </c>
-      <c r="B7" s="13" t="n">
-        <v>4</v>
-      </c>
-      <c r="C7" s="13" t="inlineStr">
-        <is>
-          <t>ESLint v9 config rozbitý</t>
-        </is>
-      </c>
-      <c r="D7" s="13" t="inlineStr">
-        <is>
-          <t>Daniela</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="32" customHeight="1">
+          <t>až 3 000 000</t>
+        </is>
+      </c>
+      <c r="E5" s="13" t="inlineStr">
+        <is>
+          <t>Mária (E010) + Katarína</t>
+        </is>
+      </c>
+      <c r="F5" s="13" t="inlineStr">
+        <is>
+          <t>AKTÍVNE — okamžite</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="40" customHeight="1">
+      <c r="A6" s="10" t="inlineStr">
+        <is>
+          <t>A3</t>
+        </is>
+      </c>
+      <c r="B6" s="10" t="inlineStr">
+        <is>
+          <t>GDPR čl. 17 + ZOOÚ § 23</t>
+        </is>
+      </c>
+      <c r="C6" s="10" t="inlineStr">
+        <is>
+          <t>GDPR erasure endpoint nemaže žiadne dáta</t>
+        </is>
+      </c>
+      <c r="D6" s="10" t="inlineStr">
+        <is>
+          <t>až 4% obratu (€40k-400k)</t>
+        </is>
+      </c>
+      <c r="E6" s="10" t="inlineStr">
+        <is>
+          <t>Katarína + Petra (E006)</t>
+        </is>
+      </c>
+      <c r="F6" s="10" t="inlineStr">
+        <is>
+          <t>30-dňová lehota plynie</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="40" customHeight="1">
+      <c r="A7" s="10" t="inlineStr">
+        <is>
+          <t>A4</t>
+        </is>
+      </c>
+      <c r="B7" s="10" t="inlineStr">
+        <is>
+          <t>AML zákon 297/2008 § 10</t>
+        </is>
+      </c>
+      <c r="C7" s="10" t="inlineStr">
+        <is>
+          <t>AML check pred KZ nikde nie je enforced</t>
+        </is>
+      </c>
+      <c r="D7" s="10" t="inlineStr">
+        <is>
+          <t>až 1 000 000</t>
+        </is>
+      </c>
+      <c r="E7" s="10" t="inlineStr">
+        <is>
+          <t>Lenka (E008) + Katarína</t>
+        </is>
+      </c>
+      <c r="F7" s="10" t="inlineStr">
+        <is>
+          <t>2 týždne</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="40" customHeight="1">
       <c r="A8" s="13" t="inlineStr">
         <is>
-          <t>P0</t>
-        </is>
-      </c>
-      <c r="B8" s="13" t="n">
-        <v>5</v>
+          <t>A5</t>
+        </is>
+      </c>
+      <c r="B8" s="13" t="inlineStr">
+        <is>
+          <t>Zákon o ERP 289/2008 § 17</t>
+        </is>
       </c>
       <c r="C8" s="13" t="inlineStr">
         <is>
-          <t>ai_usage_log tabuľka chýba</t>
+          <t>eKasa pre RKty od 1.1.2026 — žiadna integrácia</t>
         </is>
       </c>
       <c r="D8" s="13" t="inlineStr">
         <is>
-          <t>Eva + Mária</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="32" customHeight="1">
+          <t>až 20 000 + zákaz</t>
+        </is>
+      </c>
+      <c r="E8" s="13" t="inlineStr">
+        <is>
+          <t>Mária + Katarína</t>
+        </is>
+      </c>
+      <c r="F8" s="13" t="inlineStr">
+        <is>
+          <t>AKTÍVNE — okamžite</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="40" customHeight="1">
       <c r="A9" s="10" t="inlineStr">
         <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="B9" s="10" t="n">
-        <v>6</v>
+          <t>A6</t>
+        </is>
+      </c>
+      <c r="B9" s="10" t="inlineStr">
+        <is>
+          <t>DPH § 27 ods. 1</t>
+        </is>
       </c>
       <c r="C9" s="10" t="inlineStr">
         <is>
-          <t>Pagination na list endpointoch (scale 100 maklerov)</t>
+          <t>DPH sadzba 23% od 1.1.2026 — nikde v code</t>
         </is>
       </c>
       <c r="D9" s="10" t="inlineStr">
         <is>
-          <t>Michal koord</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="32" customHeight="1">
+          <t>2 000–10 000 per faktúra</t>
+        </is>
+      </c>
+      <c r="E9" s="10" t="inlineStr">
+        <is>
+          <t>Mária + dev</t>
+        </is>
+      </c>
+      <c r="F9" s="10" t="inlineStr">
+        <is>
+          <t>mesiac</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="40" customHeight="1">
       <c r="A10" s="10" t="inlineStr">
         <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="B10" s="10" t="n">
-        <v>7</v>
+          <t>A7</t>
+        </is>
+      </c>
+      <c r="B10" s="10" t="inlineStr">
+        <is>
+          <t>GDPR čl. 5 ods. 2 + ZOOÚ § 31</t>
+        </is>
       </c>
       <c r="C10" s="10" t="inlineStr">
         <is>
-          <t>Materialized views pre /manazer dashboard</t>
+          <t>Audit log iba 3.6% (5/137 routes)</t>
         </is>
       </c>
       <c r="D10" s="10" t="inlineStr">
         <is>
-          <t>Patrik + Michal</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="32" customHeight="1">
+          <t>až 4% obratu</t>
+        </is>
+      </c>
+      <c r="E10" s="10" t="inlineStr">
+        <is>
+          <t>Katarína + všetci TL</t>
+        </is>
+      </c>
+      <c r="F10" s="10" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="40" customHeight="1">
       <c r="A11" s="10" t="inlineStr">
         <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="B11" s="10" t="n">
-        <v>8</v>
+          <t>A8</t>
+        </is>
+      </c>
+      <c r="B11" s="10" t="inlineStr">
+        <is>
+          <t>DPH § 71 ods. 1 písm. b</t>
+        </is>
       </c>
       <c r="C11" s="10" t="inlineStr">
         <is>
-          <t>AML hard blocker pred KZ podpis</t>
+          <t>Faktúra číslovanie nemá UNIQUE constraint v DB</t>
         </is>
       </c>
       <c r="D11" s="10" t="inlineStr">
         <is>
-          <t>Lenka + Katarína</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="32" customHeight="1">
+          <t>1 000–5 000 + správa nesúl.</t>
+        </is>
+      </c>
+      <c r="E11" s="10" t="inlineStr">
+        <is>
+          <t>Mária + dev</t>
+        </is>
+      </c>
+      <c r="F11" s="10" t="inlineStr">
+        <is>
+          <t>mesiac</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="40" customHeight="1">
       <c r="A12" s="10" t="inlineStr">
         <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="B12" s="10" t="n">
-        <v>9</v>
+          <t>A9</t>
+        </is>
+      </c>
+      <c r="B12" s="10" t="inlineStr">
+        <is>
+          <t>GDPR čl. 28</t>
+        </is>
       </c>
       <c r="C12" s="10" t="inlineStr">
         <is>
-          <t>Reconnect Google OAuth UX</t>
+          <t>DPA s 10 vendormi — checklist a status TBD</t>
         </is>
       </c>
       <c r="D12" s="10" t="inlineStr">
         <is>
-          <t>Roman</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="32" customHeight="1">
+          <t>až 2% obratu</t>
+        </is>
+      </c>
+      <c r="E12" s="10" t="inlineStr">
+        <is>
+          <t>Pavol (E026) + Katarína</t>
+        </is>
+      </c>
+      <c r="F12" s="10" t="inlineStr">
+        <is>
+          <t>2 mesiace</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="40" customHeight="1">
       <c r="A13" s="10" t="inlineStr">
         <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="B13" s="10" t="n">
-        <v>10</v>
+          <t>A10</t>
+        </is>
+      </c>
+      <c r="B13" s="10" t="inlineStr">
+        <is>
+          <t>LP/2025/305 (nový ZOOÚ)</t>
+        </is>
       </c>
       <c r="C13" s="10" t="inlineStr">
         <is>
-          <t>30-day device verification</t>
+          <t>Rodné číslo zákaz zverejnenia (od 1.1.2027)</t>
         </is>
       </c>
       <c r="D13" s="10" t="inlineStr">
         <is>
-          <t>Lukáš</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="32" customHeight="1">
+          <t>až 10 000 000</t>
+        </is>
+      </c>
+      <c r="E13" s="10" t="inlineStr">
+        <is>
+          <t>Adam + Katarína</t>
+        </is>
+      </c>
+      <c r="F13" s="10" t="inlineStr">
+        <is>
+          <t>pred 1.1.2027</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="40" customHeight="1">
       <c r="A14" s="10" t="inlineStr">
         <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="B14" s="10" t="n">
-        <v>11</v>
+          <t>A11</t>
+        </is>
+      </c>
+      <c r="B14" s="10" t="inlineStr">
+        <is>
+          <t>GDPR čl. 33</t>
+        </is>
       </c>
       <c r="C14" s="10" t="inlineStr">
         <is>
-          <t>GitHub Actions CI/CD (TS+test+audit gate)</t>
+          <t>Breach notification 72h playbook neexistuje</t>
         </is>
       </c>
       <c r="D14" s="10" t="inlineStr">
         <is>
-          <t>Jaroslav</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="32" customHeight="1">
+          <t>až 4% obratu</t>
+        </is>
+      </c>
+      <c r="E14" s="10" t="inlineStr">
+        <is>
+          <t>Adam + Katarína</t>
+        </is>
+      </c>
+      <c r="F14" s="10" t="inlineStr">
+        <is>
+          <t>2 mesiace</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="40" customHeight="1">
       <c r="A15" s="10" t="inlineStr">
         <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="B15" s="10" t="n">
-        <v>12</v>
+          <t>A12</t>
+        </is>
+      </c>
+      <c r="B15" s="10" t="inlineStr">
+        <is>
+          <t>Vnútorná policy</t>
+        </is>
       </c>
       <c r="C15" s="10" t="inlineStr">
         <is>
-          <t>Cron health monitoring tabuľka cron_runs</t>
+          <t>Retention cron pre audit_log &gt;90d</t>
         </is>
       </c>
       <c r="D15" s="10" t="inlineStr">
         <is>
-          <t>Patrik</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="32" customHeight="1">
-      <c r="A16" s="10" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="B16" s="10" t="n">
-        <v>13</v>
-      </c>
-      <c r="C16" s="10" t="inlineStr">
-        <is>
-          <t>Password validation min 12+complexity register/reset</t>
-        </is>
-      </c>
-      <c r="D16" s="10" t="inlineStr">
-        <is>
-          <t>Lukáš</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="32" customHeight="1">
-      <c r="A17" s="10" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="B17" s="10" t="n">
-        <v>14</v>
-      </c>
-      <c r="C17" s="10" t="inlineStr">
-        <is>
-          <t>Brand voice blacklist v AI Writer pre-display</t>
-        </is>
-      </c>
-      <c r="D17" s="10" t="inlineStr">
-        <is>
-          <t>Eva + Veronika</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="32" customHeight="1">
-      <c r="A18" s="10" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="B18" s="10" t="n">
-        <v>15</v>
-      </c>
-      <c r="C18" s="10" t="inlineStr">
-        <is>
-          <t>Test coverage pre 8 critical flows</t>
-        </is>
-      </c>
-      <c r="D18" s="10" t="inlineStr">
-        <is>
-          <t>Daniela</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="32" customHeight="1">
-      <c r="A19" s="12" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="B19" s="12" t="n">
-        <v>24</v>
-      </c>
-      <c r="C19" s="12" t="inlineStr">
-        <is>
-          <t>2FA / TOTP pre adminov</t>
-        </is>
-      </c>
-      <c r="D19" s="12" t="inlineStr">
-        <is>
-          <t>Lukáš</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="32" customHeight="1">
-      <c r="A20" s="12" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="B20" s="12" t="n">
-        <v>25</v>
-      </c>
-      <c r="C20" s="12" t="inlineStr">
-        <is>
-          <t>SWR/React Query migrácia</t>
-        </is>
-      </c>
-      <c r="D20" s="12" t="inlineStr">
-        <is>
-          <t>Michal + Tech Leads</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="32" customHeight="1">
-      <c r="A21" s="12" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="B21" s="12" t="n">
-        <v>26</v>
-      </c>
-      <c r="C21" s="12" t="inlineStr">
-        <is>
-          <t>Sec Audit: anon RLS deep scan automated</t>
-        </is>
-      </c>
-      <c r="D21" s="12" t="inlineStr">
-        <is>
-          <t>Adam</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="32" customHeight="1">
-      <c r="A22" s="12" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="B22" s="12" t="n">
-        <v>41</v>
-      </c>
-      <c r="C22" s="12" t="inlineStr">
-        <is>
-          <t>RLS sprísnenie z USING(true) na ozajstné policies</t>
-        </is>
-      </c>
-      <c r="D22" s="12" t="inlineStr">
-        <is>
-          <t>Lukáš + Adam</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="32" customHeight="1">
-      <c r="A23" s="12" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="B23" s="12" t="n">
-        <v>42</v>
-      </c>
-      <c r="C23" s="12" t="inlineStr">
-        <is>
-          <t>Read replica pre /manazer (Supabase Pro upgrade)</t>
-        </is>
-      </c>
-      <c r="D23" s="12" t="inlineStr">
-        <is>
-          <t>Michal + Jaroslav</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="32" customHeight="1">
-      <c r="A24" s="12" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="B24" s="12" t="n">
-        <v>47</v>
-      </c>
-      <c r="C24" s="12" t="inlineStr">
-        <is>
-          <t>Mobile viewport tests v Playwright</t>
-        </is>
-      </c>
-      <c r="D24" s="12" t="inlineStr">
-        <is>
-          <t>Šimon + Daniela</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="6" t="inlineStr">
-        <is>
-          <t>Stav (z memory/roadmap.md):</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>P0 open: 5  |  P1 open: 18  |  P2 open: 17  |  P3 open: 10  |  Total: 50</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>Closure rate target: ≥ 50% mesačne (Inspector General tracks)</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>Sprint review: piatok 16:00 (PM E021 Peter Halás)</t>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E15" s="10" t="inlineStr">
+        <is>
+          <t>Patrik (E013)</t>
+        </is>
+      </c>
+      <c r="F15" s="10" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A1:F1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5132,620 +6875,861 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:G33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="60" customWidth="1" min="3" max="3"/>
-    <col width="38" customWidth="1" min="4" max="4"/>
-    <col width="26" customWidth="1" min="5" max="5"/>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="38" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Denný režim — automatizované cron jobs + audit rutiny</t>
+          <t>Risk Register (20 položiek, FRM metodika)</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Čas UTC</t>
+          <t>#</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Čas SK (UTC+2)</t>
+          <t>Riziko</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Akcia</t>
+          <t>Pravdep.</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Kto vykonáva</t>
+          <t>Dopad</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Reportuje komu</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="35" customHeight="1">
-      <c r="A4" s="12" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="B4" s="12" t="inlineStr">
-        <is>
-          <t>02:00</t>
-        </is>
-      </c>
-      <c r="C4" s="12" t="inlineStr">
-        <is>
-          <t>Cleanup cron (staré audit záznamy, expired sessions)</t>
-        </is>
-      </c>
-      <c r="D4" s="12" t="inlineStr">
-        <is>
-          <t>Vercel (automatický)</t>
-        </is>
-      </c>
-      <c r="E4" s="12" t="inlineStr">
-        <is>
-          <t>E017 Jaroslav (DevOps)</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="35" customHeight="1">
-      <c r="A5" s="12" t="inlineStr">
-        <is>
-          <t>01:00</t>
-        </is>
-      </c>
-      <c r="B5" s="12" t="inlineStr">
-        <is>
-          <t>03:00</t>
-        </is>
-      </c>
-      <c r="C5" s="12" t="inlineStr">
-        <is>
-          <t>Pravidelné náklady — auto-pridanie do prehľadu (0–2 dni pred splatnosťou)</t>
-        </is>
-      </c>
-      <c r="D5" s="12" t="inlineStr">
-        <is>
-          <t>Vercel cron</t>
-        </is>
-      </c>
-      <c r="E5" s="12" t="inlineStr">
-        <is>
-          <t>E010 Mária (Financie)</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="35" customHeight="1">
-      <c r="A6" s="12" t="inlineStr">
-        <is>
-          <t>02:00</t>
-        </is>
-      </c>
-      <c r="B6" s="12" t="inlineStr">
-        <is>
-          <t>04:00</t>
-        </is>
-      </c>
-      <c r="C6" s="12" t="inlineStr">
-        <is>
-          <t>Domain audits — všetkých 10 modulov (audit-security.sh, audit-monitor.sh, atď.)</t>
-        </is>
-      </c>
-      <c r="D6" s="12" t="inlineStr">
-        <is>
-          <t>10 Tech Leads (E004-E013)</t>
-        </is>
-      </c>
-      <c r="E6" s="12" t="inlineStr">
-        <is>
-          <t>E003 Tomáš (CTO)</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="35" customHeight="1">
+          <t>Skóre</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Mitigácia</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="32" customHeight="1">
+      <c r="A4" s="10" t="inlineStr">
+        <is>
+          <t>O1</t>
+        </is>
+      </c>
+      <c r="B4" s="10" t="inlineStr">
+        <is>
+          <t>Cron silent fail (Monitor 8d incident)</t>
+        </is>
+      </c>
+      <c r="C4" s="10" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D4" s="10" t="inlineStr">
+        <is>
+          <t>Stredný (insights)</t>
+        </is>
+      </c>
+      <c r="E4" s="10" t="inlineStr">
+        <is>
+          <t>15 HIGH</t>
+        </is>
+      </c>
+      <c r="F4" s="10" t="inlineStr">
+        <is>
+          <t>Patrik+Martin</t>
+        </is>
+      </c>
+      <c r="G4" s="10" t="inlineStr">
+        <is>
+          <t>cron_runs + healthcheck &gt;36h</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="32" customHeight="1">
+      <c r="A5" s="10" t="inlineStr">
+        <is>
+          <t>O2</t>
+        </is>
+      </c>
+      <c r="B5" s="10" t="inlineStr">
+        <is>
+          <t>Vercel platform outage</t>
+        </is>
+      </c>
+      <c r="C5" s="10" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="D5" s="10" t="inlineStr">
+        <is>
+          <t>Vysoký (0€ revenue)</t>
+        </is>
+      </c>
+      <c r="E5" s="10" t="inlineStr">
+        <is>
+          <t>10 HIGH</t>
+        </is>
+      </c>
+      <c r="F5" s="10" t="inlineStr">
+        <is>
+          <t>Jaroslav</t>
+        </is>
+      </c>
+      <c r="G5" s="10" t="inlineStr">
+        <is>
+          <t>SLA escalation, status subscribe</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="32" customHeight="1">
+      <c r="A6" s="10" t="inlineStr">
+        <is>
+          <t>O3</t>
+        </is>
+      </c>
+      <c r="B6" s="10" t="inlineStr">
+        <is>
+          <t>Supabase data loss / outage</t>
+        </is>
+      </c>
+      <c r="C6" s="10" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="D6" s="10" t="inlineStr">
+        <is>
+          <t>CATASTROFICKÝ</t>
+        </is>
+      </c>
+      <c r="E6" s="10" t="inlineStr">
+        <is>
+          <t>15 HIGH</t>
+        </is>
+      </c>
+      <c r="F6" s="10" t="inlineStr">
+        <is>
+          <t>Jaroslav+Michal</t>
+        </is>
+      </c>
+      <c r="G6" s="10" t="inlineStr">
+        <is>
+          <t>Daily pg_dump→S3+Drive, drill</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="32" customHeight="1">
       <c r="A7" s="12" t="inlineStr">
         <is>
-          <t>03:00</t>
+          <t>O4</t>
         </is>
       </c>
       <c r="B7" s="12" t="inlineStr">
         <is>
-          <t>05:00</t>
+          <t>Single person dependency</t>
         </is>
       </c>
       <c r="C7" s="12" t="inlineStr">
         <is>
-          <t>QA audit — test coverage report, regression status</t>
+          <t>MED</t>
         </is>
       </c>
       <c r="D7" s="12" t="inlineStr">
         <is>
-          <t>E014 Daniela</t>
+          <t>Stredný</t>
         </is>
       </c>
       <c r="E7" s="12" t="inlineStr">
         <is>
-          <t>E003 Tomáš (CTO)</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="35" customHeight="1">
+          <t>9 MED</t>
+        </is>
+      </c>
+      <c r="F7" s="12" t="inlineStr">
+        <is>
+          <t>HR (TBD) + COO</t>
+        </is>
+      </c>
+      <c r="G7" s="12" t="inlineStr">
+        <is>
+          <t>Cross-training, runbooks</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="32" customHeight="1">
       <c r="A8" s="12" t="inlineStr">
         <is>
-          <t>03:30</t>
+          <t>O5</t>
         </is>
       </c>
       <c r="B8" s="12" t="inlineStr">
         <is>
-          <t>05:30</t>
+          <t>API key rotation chyba (Resend, AI)</t>
         </is>
       </c>
       <c r="C8" s="12" t="inlineStr">
         <is>
-          <t>SRE perf benchmark — response time check kritických endpointov</t>
+          <t>MED</t>
         </is>
       </c>
       <c r="D8" s="12" t="inlineStr">
         <is>
-          <t>E015 Michal</t>
+          <t>Stredný</t>
         </is>
       </c>
       <c r="E8" s="12" t="inlineStr">
         <is>
-          <t>E003 Tomáš (CTO)</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="35" customHeight="1">
-      <c r="A9" s="12" t="inlineStr">
-        <is>
-          <t>04:00</t>
-        </is>
-      </c>
-      <c r="B9" s="12" t="inlineStr">
-        <is>
-          <t>06:00</t>
-        </is>
-      </c>
-      <c r="C9" s="12" t="inlineStr">
-        <is>
-          <t>Security deep scan (PONDELOK týždenne) — anon RLS leak, env audit, pen-test scenáre</t>
-        </is>
-      </c>
-      <c r="D9" s="12" t="inlineStr">
-        <is>
-          <t>E016 Adam (Sec Auditor)</t>
-        </is>
-      </c>
-      <c r="E9" s="12" t="inlineStr">
-        <is>
-          <t>E001 Aleš (CEO)</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="35" customHeight="1">
-      <c r="A10" s="12" t="inlineStr">
-        <is>
-          <t>05:00</t>
-        </is>
-      </c>
-      <c r="B10" s="12" t="inlineStr">
-        <is>
-          <t>07:00</t>
-        </is>
-      </c>
-      <c r="C10" s="12" t="inlineStr">
-        <is>
-          <t>Compliance check — GDPR coverage, audit log integrity, faktúra sequence</t>
-        </is>
-      </c>
-      <c r="D10" s="12" t="inlineStr">
-        <is>
-          <t>E018 Katarína</t>
-        </is>
-      </c>
-      <c r="E10" s="12" t="inlineStr">
-        <is>
-          <t>E001 Aleš (CEO)</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="35" customHeight="1">
+          <t>9 MED</t>
+        </is>
+      </c>
+      <c r="F8" s="12" t="inlineStr">
+        <is>
+          <t>Jaroslav</t>
+        </is>
+      </c>
+      <c r="G8" s="12" t="inlineStr">
+        <is>
+          <t>90d rotation kalendár</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="32" customHeight="1">
+      <c r="A9" s="10" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="B9" s="10" t="inlineStr">
+        <is>
+          <t>AI cost runaway (parse-doc loop)</t>
+        </is>
+      </c>
+      <c r="C9" s="10" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D9" s="10" t="inlineStr">
+        <is>
+          <t>5-50k€/mes</t>
+        </is>
+      </c>
+      <c r="E9" s="10" t="inlineStr">
+        <is>
+          <t>15 HIGH</t>
+        </is>
+      </c>
+      <c r="F9" s="10" t="inlineStr">
+        <is>
+          <t>Eva+Mária</t>
+        </is>
+      </c>
+      <c r="G9" s="10" t="inlineStr">
+        <is>
+          <t>ai_usage_log, alert &gt;50€/d</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="32" customHeight="1">
+      <c r="A10" s="10" t="inlineStr">
+        <is>
+          <t>F2</t>
+        </is>
+      </c>
+      <c r="B10" s="10" t="inlineStr">
+        <is>
+          <t>Faktúra číslovanie duplicit/skip</t>
+        </is>
+      </c>
+      <c r="C10" s="10" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="D10" s="10" t="inlineStr">
+        <is>
+          <t>Vysoký (daň pokuta)</t>
+        </is>
+      </c>
+      <c r="E10" s="10" t="inlineStr">
+        <is>
+          <t>10 HIGH</t>
+        </is>
+      </c>
+      <c r="F10" s="10" t="inlineStr">
+        <is>
+          <t>Mária+dev</t>
+        </is>
+      </c>
+      <c r="G10" s="10" t="inlineStr">
+        <is>
+          <t>Atomic SQL sequence</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="32" customHeight="1">
       <c r="A11" s="12" t="inlineStr">
         <is>
-          <t>05:00</t>
+          <t>F3</t>
         </is>
       </c>
       <c r="B11" s="12" t="inlineStr">
         <is>
-          <t>07:00</t>
+          <t>Provízia spor (klient nezaplatí)</t>
         </is>
       </c>
       <c r="C11" s="12" t="inlineStr">
         <is>
-          <t>Volni klienti cron — 24h dropoff klientov bez aktivity</t>
+          <t>MED</t>
         </is>
       </c>
       <c r="D11" s="12" t="inlineStr">
         <is>
-          <t>Vercel cron</t>
+          <t>1-10k€/spor</t>
         </is>
       </c>
       <c r="E11" s="12" t="inlineStr">
         <is>
-          <t>E006 Petra (Klienti)</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="35" customHeight="1">
+          <t>9 MED</t>
+        </is>
+      </c>
+      <c r="F11" s="12" t="inlineStr">
+        <is>
+          <t>Mária+Katarína</t>
+        </is>
+      </c>
+      <c r="G11" s="12" t="inlineStr">
+        <is>
+          <t>Audit log + e-podpis</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="32" customHeight="1">
       <c r="A12" s="12" t="inlineStr">
         <is>
-          <t>06:00</t>
+          <t>F4</t>
         </is>
       </c>
       <c r="B12" s="12" t="inlineStr">
         <is>
-          <t>08:00</t>
+          <t>Cashflow gap (klient 60-90d po KZ)</t>
         </is>
       </c>
       <c r="C12" s="12" t="inlineStr">
         <is>
-          <t>API status cron — healthcheck 3rd party (Anthropic, Gemini, Google, Resend)</t>
+          <t>MED</t>
         </is>
       </c>
       <c r="D12" s="12" t="inlineStr">
         <is>
-          <t>Vercel cron</t>
+          <t>Stredný (100k+ outstanding)</t>
         </is>
       </c>
       <c r="E12" s="12" t="inlineStr">
         <is>
-          <t>E015 Michal (SRE)</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="35" customHeight="1">
+          <t>9 MED</t>
+        </is>
+      </c>
+      <c r="F12" s="12" t="inlineStr">
+        <is>
+          <t>Mária</t>
+        </is>
+      </c>
+      <c r="G12" s="12" t="inlineStr">
+        <is>
+          <t>DSO tracking, T+14/T+30 upomienky</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="32" customHeight="1">
       <c r="A13" s="12" t="inlineStr">
         <is>
-          <t>06:30</t>
+          <t>F5</t>
         </is>
       </c>
       <c r="B13" s="12" t="inlineStr">
         <is>
-          <t>08:30</t>
+          <t>DPH 23% neaplikovaná v faktúre</t>
         </is>
       </c>
       <c r="C13" s="12" t="inlineStr">
         <is>
-          <t>Daily report email tebe — 'Vianema engineering daily: 8/10 green, 2 warnings'</t>
+          <t>MED</t>
         </is>
       </c>
       <c r="D13" s="12" t="inlineStr">
         <is>
-          <t>E002 Claude (orchestrator)</t>
+          <t>Stredný + €3320/faktúra</t>
         </is>
       </c>
       <c r="E13" s="12" t="inlineStr">
         <is>
-          <t>E001 Aleš (CEO)</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="35" customHeight="1">
-      <c r="A14" s="12" t="inlineStr">
-        <is>
-          <t>07:00</t>
-        </is>
-      </c>
-      <c r="B14" s="12" t="inlineStr">
-        <is>
-          <t>09:00</t>
-        </is>
-      </c>
-      <c r="C14" s="12" t="inlineStr">
-        <is>
-          <t>LV reminder cron — pripomienka pre LV-ká blízko expirácie</t>
-        </is>
-      </c>
-      <c r="D14" s="12" t="inlineStr">
-        <is>
-          <t>Vercel cron</t>
-        </is>
-      </c>
-      <c r="E14" s="12" t="inlineStr">
-        <is>
-          <t>E008 Lenka (Náberáky)</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="35" customHeight="1">
-      <c r="A15" s="12" t="inlineStr">
-        <is>
-          <t>08:00</t>
-        </is>
-      </c>
-      <c r="B15" s="12" t="inlineStr">
-        <is>
-          <t>10:00</t>
-        </is>
-      </c>
-      <c r="C15" s="12" t="inlineStr">
-        <is>
-          <t>Scrape cron (Monitor) — daily fetch z Bazos/Reality/Nehnuteľnosti</t>
-        </is>
-      </c>
-      <c r="D15" s="12" t="inlineStr">
-        <is>
-          <t>Vercel cron</t>
-        </is>
-      </c>
-      <c r="E15" s="12" t="inlineStr">
-        <is>
-          <t>E005 Martin (Monitor)</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="35" customHeight="1">
-      <c r="A16" s="12" t="inlineStr">
-        <is>
-          <t>09:00</t>
-        </is>
-      </c>
-      <c r="B16" s="12" t="inlineStr">
-        <is>
-          <t>11:00</t>
-        </is>
-      </c>
-      <c r="C16" s="12" t="inlineStr">
-        <is>
-          <t>Monitor-daily — vyhodnocovanie signálov (RELISTED, motivated sellers)</t>
-        </is>
-      </c>
-      <c r="D16" s="12" t="inlineStr">
-        <is>
-          <t>Vercel cron</t>
-        </is>
-      </c>
-      <c r="E16" s="12" t="inlineStr">
-        <is>
-          <t>E005 Martin (Monitor)</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="35" customHeight="1">
+          <t>9 MED</t>
+        </is>
+      </c>
+      <c r="F13" s="12" t="inlineStr">
+        <is>
+          <t>Mária+dev</t>
+        </is>
+      </c>
+      <c r="G13" s="12" t="inlineStr">
+        <is>
+          <t>Code audit DPH konštánt</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="32" customHeight="1">
+      <c r="A14" s="10" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
+      <c r="B14" s="10" t="inlineStr">
+        <is>
+          <t>GDPR pokuta — audit log 6% coverage</t>
+        </is>
+      </c>
+      <c r="C14" s="10" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D14" s="10" t="inlineStr">
+        <is>
+          <t>40k-400k+€</t>
+        </is>
+      </c>
+      <c r="E14" s="10" t="inlineStr">
+        <is>
+          <t>15 HIGH</t>
+        </is>
+      </c>
+      <c r="F14" s="10" t="inlineStr">
+        <is>
+          <t>Katarína</t>
+        </is>
+      </c>
+      <c r="G14" s="10" t="inlineStr">
+        <is>
+          <t>Audit log 100%, DPIA AI Writer</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="32" customHeight="1">
+      <c r="A15" s="13" t="inlineStr">
+        <is>
+          <t>C2</t>
+        </is>
+      </c>
+      <c r="B15" s="13" t="inlineStr">
+        <is>
+          <t>AML — VIANEMA neregistrovaná do 31.8.2026</t>
+        </is>
+      </c>
+      <c r="C15" s="13" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D15" s="13" t="inlineStr">
+        <is>
+          <t>165k€ + zákaz</t>
+        </is>
+      </c>
+      <c r="E15" s="13" t="inlineStr">
+        <is>
+          <t>25 CRITICAL</t>
+        </is>
+      </c>
+      <c r="F15" s="13" t="inlineStr">
+        <is>
+          <t>Katarína</t>
+        </is>
+      </c>
+      <c r="G15" s="13" t="inlineStr">
+        <is>
+          <t>Registrácia FIU SR TERAZ</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="32" customHeight="1">
+      <c r="A16" s="10" t="inlineStr">
+        <is>
+          <t>C3</t>
+        </is>
+      </c>
+      <c r="B16" s="10" t="inlineStr">
+        <is>
+          <t>eKasa nepoužívaná pri hotovostnej provízii</t>
+        </is>
+      </c>
+      <c r="C16" s="10" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D16" s="10" t="inlineStr">
+        <is>
+          <t>330-33000€ per</t>
+        </is>
+      </c>
+      <c r="E16" s="10" t="inlineStr">
+        <is>
+          <t>15 HIGH</t>
+        </is>
+      </c>
+      <c r="F16" s="10" t="inlineStr">
+        <is>
+          <t>Mária+Katarína</t>
+        </is>
+      </c>
+      <c r="G16" s="10" t="inlineStr">
+        <is>
+          <t>Policy 'iba bezhotovostné' alebo eKasa</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="32" customHeight="1">
       <c r="A17" s="12" t="inlineStr">
         <is>
-          <t>12:00</t>
+          <t>C4</t>
         </is>
       </c>
       <c r="B17" s="12" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>Faktúra retencia &lt;10y</t>
         </is>
       </c>
       <c r="C17" s="12" t="inlineStr">
         <is>
-          <t>Tím standup (async, zápis v memory/standup.md) — čo robím, čo blokuje</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="D17" s="12" t="inlineStr">
         <is>
-          <t>Všetci Tech Leads</t>
+          <t>Vysoký (daň)</t>
         </is>
       </c>
       <c r="E17" s="12" t="inlineStr">
         <is>
-          <t>E003 Tomáš (CTO)</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="35" customHeight="1">
+          <t>5 MED</t>
+        </is>
+      </c>
+      <c r="F17" s="12" t="inlineStr">
+        <is>
+          <t>Mária+Jaroslav</t>
+        </is>
+      </c>
+      <c r="G17" s="12" t="inlineStr">
+        <is>
+          <t>Backup retention 10y, Object Lock</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="32" customHeight="1">
       <c r="A18" s="12" t="inlineStr">
         <is>
-          <t>On-demand</t>
+          <t>C5</t>
         </is>
       </c>
       <c r="B18" s="12" t="inlineStr">
         <is>
-          <t>On-demand</t>
+          <t>AI automated decision bez disclosure</t>
         </is>
       </c>
       <c r="C18" s="12" t="inlineStr">
         <is>
-          <t>PR review — pred každým merge</t>
+          <t>MED</t>
         </is>
       </c>
       <c r="D18" s="12" t="inlineStr">
         <is>
-          <t>E014 Daniela + Tech Lead + (sec/brand/ux ak relevant)</t>
+          <t>Stredný-Vysoký</t>
         </is>
       </c>
       <c r="E18" s="12" t="inlineStr">
         <is>
-          <t>E002 Claude (COO)</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="35" customHeight="1">
-      <c r="A19" s="12" t="inlineStr">
-        <is>
-          <t>Týždenne</t>
-        </is>
-      </c>
-      <c r="B19" s="12" t="inlineStr">
-        <is>
-          <t>PIATOK 16:00</t>
-        </is>
-      </c>
-      <c r="C19" s="12" t="inlineStr">
-        <is>
-          <t>Sprint review + roadmap update — čo sa stalo, čo prichádza</t>
-        </is>
-      </c>
-      <c r="D19" s="12" t="inlineStr">
-        <is>
-          <t>E021 Peter (PM)</t>
-        </is>
-      </c>
-      <c r="E19" s="12" t="inlineStr">
-        <is>
-          <t>E001 Aleš (CEO)</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="35" customHeight="1">
-      <c r="A20" s="12" t="inlineStr">
-        <is>
-          <t>Mesačne</t>
-        </is>
-      </c>
-      <c r="B20" s="12" t="inlineStr">
-        <is>
-          <t>1. v mesiaci</t>
-        </is>
-      </c>
-      <c r="C20" s="12" t="inlineStr">
-        <is>
-          <t>Faktúra integrity audit — duplicit, sequence, daň, splatnosť</t>
-        </is>
-      </c>
-      <c r="D20" s="12" t="inlineStr">
-        <is>
-          <t>E010 Mária + E018 Katarína</t>
-        </is>
-      </c>
-      <c r="E20" s="12" t="inlineStr">
-        <is>
-          <t>E001 Aleš (CEO)</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="35" customHeight="1">
+          <t>9 MED</t>
+        </is>
+      </c>
+      <c r="F18" s="12" t="inlineStr">
+        <is>
+          <t>Katarína+Eva</t>
+        </is>
+      </c>
+      <c r="G18" s="12" t="inlineStr">
+        <is>
+          <t>Privacy AI sekcia, opt-out, DPIA</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="32" customHeight="1">
+      <c r="A19" s="10" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="B19" s="10" t="inlineStr">
+        <is>
+          <t>Klient PII leak (anon RLS USING(true))</t>
+        </is>
+      </c>
+      <c r="C19" s="10" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D19" s="10" t="inlineStr">
+        <is>
+          <t>CATASTROFICKÝ</t>
+        </is>
+      </c>
+      <c r="E19" s="10" t="inlineStr">
+        <is>
+          <t>15 HIGH</t>
+        </is>
+      </c>
+      <c r="F19" s="10" t="inlineStr">
+        <is>
+          <t>Adam+Lukáš</t>
+        </is>
+      </c>
+      <c r="G19" s="10" t="inlineStr">
+        <is>
+          <t>Systematický scan + sprísnenie</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="32" customHeight="1">
+      <c r="A20" s="10" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B20" s="10" t="inlineStr">
+        <is>
+          <t>Maklér phishing → kompromis CRM</t>
+        </is>
+      </c>
+      <c r="C20" s="10" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D20" s="10" t="inlineStr">
+        <is>
+          <t>Vysoký (multi-tenant)</t>
+        </is>
+      </c>
+      <c r="E20" s="10" t="inlineStr">
+        <is>
+          <t>15 HIGH</t>
+        </is>
+      </c>
+      <c r="F20" s="10" t="inlineStr">
+        <is>
+          <t>Adam+Lukáš</t>
+        </is>
+      </c>
+      <c r="G20" s="10" t="inlineStr">
+        <is>
+          <t>2FA admin, 30d device verify</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="32" customHeight="1">
       <c r="A21" s="12" t="inlineStr">
         <is>
-          <t>Kvartálne</t>
+          <t>R3</t>
         </is>
       </c>
       <c r="B21" s="12" t="inlineStr">
         <is>
-          <t>1. deň kvartálu</t>
+          <t>Resend/IP spam blacklist</t>
         </is>
       </c>
       <c r="C21" s="12" t="inlineStr">
         <is>
-          <t>Security health report — známkovanie všetkých 10 domén</t>
+          <t>MED</t>
         </is>
       </c>
       <c r="D21" s="12" t="inlineStr">
         <is>
-          <t>E016 Adam (Sec Auditor)</t>
+          <t>Stredný (emaily fail)</t>
         </is>
       </c>
       <c r="E21" s="12" t="inlineStr">
         <is>
-          <t>E001 Aleš (CEO)</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="35" customHeight="1">
-      <c r="A22" s="15" t="inlineStr">
-        <is>
-          <t>01:30</t>
-        </is>
-      </c>
-      <c r="B22" s="15" t="inlineStr">
-        <is>
-          <t>03:30</t>
-        </is>
-      </c>
-      <c r="C22" s="15" t="inlineStr">
-        <is>
-          <t>Meta audit (memory rot, audit script freshness) — Inspector General</t>
-        </is>
-      </c>
-      <c r="D22" s="15" t="inlineStr">
-        <is>
-          <t>E023 Mária (IG)</t>
-        </is>
-      </c>
-      <c r="E22" s="15" t="inlineStr">
-        <is>
-          <t>E002 Claude (COO)</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="35" customHeight="1">
-      <c r="A23" s="15" t="inlineStr">
-        <is>
-          <t>Týždenne</t>
-        </is>
-      </c>
-      <c r="B23" s="15" t="inlineStr">
-        <is>
-          <t>PIATOK 17:00</t>
-        </is>
-      </c>
-      <c r="C23" s="15" t="inlineStr">
-        <is>
-          <t>Internal audit report — kto nerobí svoju prácu, TODO trends, kritické nálezy</t>
-        </is>
-      </c>
-      <c r="D23" s="15" t="inlineStr">
-        <is>
-          <t>E023 Mária (IG)</t>
-        </is>
-      </c>
-      <c r="E23" s="15" t="inlineStr">
-        <is>
-          <t>E001 Aleš (CEO)</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="35" customHeight="1">
-      <c r="A24" s="15" t="inlineStr">
-        <is>
-          <t>Mesačne</t>
-        </is>
-      </c>
-      <c r="B24" s="15" t="inlineStr">
-        <is>
-          <t>1. v mesiaci</t>
-        </is>
-      </c>
-      <c r="C24" s="15" t="inlineStr">
-        <is>
-          <t>Aggregate external watch sources reports (čo nové v práve, security, AI atď.)</t>
-        </is>
-      </c>
-      <c r="D24" s="15" t="inlineStr">
-        <is>
-          <t>E023 + Katarína + Adam + ostatní</t>
-        </is>
-      </c>
-      <c r="E24" s="15" t="inlineStr">
-        <is>
-          <t>E001 Aleš (CEO)</t>
+          <t>9 MED</t>
+        </is>
+      </c>
+      <c r="F21" s="12" t="inlineStr">
+        <is>
+          <t>Jaroslav</t>
+        </is>
+      </c>
+      <c r="G21" s="12" t="inlineStr">
+        <is>
+          <t>DKIM/SPF/DMARC monitoring</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="32" customHeight="1">
+      <c r="A22" s="12" t="inlineStr">
+        <is>
+          <t>R4</t>
+        </is>
+      </c>
+      <c r="B22" s="12" t="inlineStr">
+        <is>
+          <t>Maklér fraud (fake faktúra)</t>
+        </is>
+      </c>
+      <c r="C22" s="12" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="D22" s="12" t="inlineStr">
+        <is>
+          <t>Vysoký</t>
+        </is>
+      </c>
+      <c r="E22" s="12" t="inlineStr">
+        <is>
+          <t>5 MED</t>
+        </is>
+      </c>
+      <c r="F22" s="12" t="inlineStr">
+        <is>
+          <t>Mária+Katarína</t>
+        </is>
+      </c>
+      <c r="G22" s="12" t="inlineStr">
+        <is>
+          <t>Approval workflow &gt;5k€</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="32" customHeight="1">
+      <c r="A23" s="12" t="inlineStr">
+        <is>
+          <t>R5</t>
+        </is>
+      </c>
+      <c r="B23" s="12" t="inlineStr">
+        <is>
+          <t>Social media / fake reviews</t>
+        </is>
+      </c>
+      <c r="C23" s="12" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D23" s="12" t="inlineStr">
+        <is>
+          <t>Stredný (SEO)</t>
+        </is>
+      </c>
+      <c r="E23" s="12" t="inlineStr">
+        <is>
+          <t>9 MED</t>
+        </is>
+      </c>
+      <c r="F23" s="12" t="inlineStr">
+        <is>
+          <t>Veronika (Brand)</t>
+        </is>
+      </c>
+      <c r="G23" s="12" t="inlineStr">
+        <is>
+          <t>Mention/Brand24, reply 24h</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="6" t="inlineStr">
+        <is>
+          <t>TOP 3 priority hneď:</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" s="7" t="inlineStr">
+        <is>
+          <t>C2 — AML registrácia (25 CRITICAL, deadline 31.8.2026, T-103 dní)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" s="7" t="inlineStr">
+        <is>
+          <t>C1 — Audit log 100% (15 HIGH, 4% revenue penalty pri ÚOOÚ)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" s="7" t="inlineStr">
+        <is>
+          <t>F1+R1 combo — AI cost runaway + PII leak (15×2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="6" t="inlineStr">
+        <is>
+          <t>Insurance plán:</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" s="7" t="inlineStr">
+        <is>
+          <t>Cyber liability — Allianz CyberRisk (~3-8k€/r) cez broker MARSH/Aon</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="B32" s="7" t="inlineStr">
+        <is>
+          <t>D&amp;O — Generali/Colonnade (2-5k€/r)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" s="7" t="inlineStr">
+        <is>
+          <t>Professional Indemnity — Wüstenrot/NN (1-3k€/r)</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A1:G1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>